<commit_message>
chore: 更新 EVP 数据产物 — 新配置 (CAP_BO1×2.5 + LEN×1.8) 重算 Step2/Step3
- Step2 全局统计: mean=1.1142 std=2.5100 (255 赛事, 15841 选手)
- Step3 重建 254 赛事 EVP 汇总 + 透视表 (含金量子表)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/event/1608/event_1608_evp_summary.xlsx
+++ b/database/event/1608/event_1608_evp_summary.xlsx
@@ -502,7 +502,7 @@
         <v>0.9883999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>1.77</v>
+        <v>1.7172</v>
       </c>
       <c r="E2" t="n">
         <v>5.4244</v>
@@ -548,7 +548,7 @@
         <v>0.6828</v>
       </c>
       <c r="D3" t="n">
-        <v>1.0925</v>
+        <v>1.0491</v>
       </c>
       <c r="E3" t="n">
         <v>3.7474</v>
@@ -594,7 +594,7 @@
         <v>0.6623</v>
       </c>
       <c r="D4" t="n">
-        <v>1.0471</v>
+        <v>1.0043</v>
       </c>
       <c r="E4" t="n">
         <v>3.635</v>
@@ -640,7 +640,7 @@
         <v>0.6068</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9241</v>
+        <v>0.883</v>
       </c>
       <c r="E5" t="n">
         <v>3.3305</v>
@@ -686,7 +686,7 @@
         <v>0.5632</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8274</v>
+        <v>0.7876</v>
       </c>
       <c r="E6" t="n">
         <v>3.0912</v>
@@ -732,7 +732,7 @@
         <v>0.2012</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0248</v>
+        <v>-0.0039</v>
       </c>
       <c r="E7" t="n">
         <v>1.1044</v>
@@ -778,7 +778,7 @@
         <v>0.0626</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.2825</v>
+        <v>-0.307</v>
       </c>
       <c r="E8" t="n">
         <v>0.3437</v>
@@ -824,7 +824,7 @@
         <v>0.0574</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.294</v>
+        <v>-0.3183</v>
       </c>
       <c r="E9" t="n">
         <v>0.3153</v>
@@ -870,7 +870,7 @@
         <v>0.0525</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.3049</v>
+        <v>-0.329</v>
       </c>
       <c r="E10" t="n">
         <v>0.2884</v>
@@ -916,7 +916,7 @@
         <v>0.0485</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.3137</v>
+        <v>-0.3378</v>
       </c>
       <c r="E11" t="n">
         <v>0.2664</v>
@@ -962,7 +962,7 @@
         <v>0.0012</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.4186</v>
+        <v>-0.4412</v>
       </c>
       <c r="E12" t="n">
         <v>0.0068</v>
@@ -1008,7 +1008,7 @@
         <v>-0.0133</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.4509</v>
+        <v>-0.4731</v>
       </c>
       <c r="E13" t="n">
         <v>-0.0732</v>
@@ -1054,7 +1054,7 @@
         <v>-0.0372</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.5038</v>
+        <v>-0.5252</v>
       </c>
       <c r="E14" t="n">
         <v>-0.2041</v>
@@ -1100,7 +1100,7 @@
         <v>-0.1273</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.7036</v>
+        <v>-0.7222</v>
       </c>
       <c r="E15" t="n">
         <v>-0.6986</v>
@@ -1146,7 +1146,7 @@
         <v>-0.1889</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.8401999999999999</v>
+        <v>-0.857</v>
       </c>
       <c r="E16" t="n">
         <v>-1.0369</v>
@@ -1192,7 +1192,7 @@
         <v>-0.2256</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.9215</v>
+        <v>-0.9372</v>
       </c>
       <c r="E17" t="n">
         <v>-1.2381</v>
@@ -1238,7 +1238,7 @@
         <v>-0.2656</v>
       </c>
       <c r="D18" t="n">
-        <v>-1.0103</v>
+        <v>-1.0247</v>
       </c>
       <c r="E18" t="n">
         <v>-1.4578</v>
@@ -1284,7 +1284,7 @@
         <v>-0.2912</v>
       </c>
       <c r="D19" t="n">
-        <v>-1.0671</v>
+        <v>-1.0807</v>
       </c>
       <c r="E19" t="n">
         <v>-1.5984</v>
@@ -1330,7 +1330,7 @@
         <v>-0.3403</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.1758</v>
+        <v>-1.1879</v>
       </c>
       <c r="E20" t="n">
         <v>-1.8674</v>
@@ -1376,7 +1376,7 @@
         <v>-0.5817</v>
       </c>
       <c r="D21" t="n">
-        <v>-1.7111</v>
+        <v>-1.7158</v>
       </c>
       <c r="E21" t="n">
         <v>-3.1925</v>

</xml_diff>

<commit_message>
feat: EVP 定案写回 — gen24 局部精调 obj=158.11 (+1.89 over seed50)
- 42 维 ±30% 邻域精调 (seed50 出发, sigma0=0.1), gen24 中断时 best 定案
- 成绩: ordered 66.7% (212/318) / in_topn 85.2% (1526/1791) / mvp 204/254 / mismatch 258.9
- W_MIS=0.1 口径演进: 基线 150.76 → seed50 156.22 → refine 158.11 (全面小幅改善, 非 trade-off)
- 重算 Step2/Step3: 255 赛事 global_stats + 254 赛事 evp_summary + 全局透视总表

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/event/1608/event_1608_evp_summary.xlsx
+++ b/database/event/1608/event_1608_evp_summary.xlsx
@@ -496,31 +496,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.4244</v>
+        <v>5.8247</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9883999999999999</v>
+        <v>1.0613</v>
       </c>
       <c r="D2" t="n">
-        <v>1.7172</v>
+        <v>1.9915</v>
       </c>
       <c r="E2" t="n">
-        <v>5.4244</v>
+        <v>5.8247</v>
       </c>
       <c r="F2" t="n">
-        <v>1.3518</v>
+        <v>2.2893</v>
       </c>
       <c r="G2" t="n">
-        <v>4.0726</v>
+        <v>3.5354</v>
       </c>
       <c r="H2" t="n">
-        <v>1.3518</v>
+        <v>2.5797</v>
       </c>
       <c r="I2" t="n">
-        <v>1.0957</v>
+        <v>1.3413</v>
       </c>
       <c r="J2" t="n">
-        <v>4.0726</v>
+        <v>3.5354</v>
       </c>
       <c r="K2" t="n">
         <v>151</v>
@@ -529,7 +529,7 @@
         <v>131</v>
       </c>
       <c r="M2" t="n">
-        <v>5.1683</v>
+        <v>4.8767</v>
       </c>
       <c r="N2" t="n">
         <v>282</v>
@@ -538,127 +538,127 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>KRIMZ</t>
+          <t>allu</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.7474</v>
+        <v>4.0961</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6828</v>
+        <v>0.7463</v>
       </c>
       <c r="D3" t="n">
-        <v>1.0491</v>
+        <v>1.2112</v>
       </c>
       <c r="E3" t="n">
-        <v>3.7474</v>
+        <v>4.0961</v>
       </c>
       <c r="F3" t="n">
-        <v>4.3422</v>
+        <v>2.4452</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.5948</v>
+        <v>1.6509</v>
       </c>
       <c r="H3" t="n">
-        <v>4.9093</v>
+        <v>3.1289</v>
       </c>
       <c r="I3" t="n">
-        <v>3.9791</v>
+        <v>1.6269</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.5948</v>
+        <v>1.6509</v>
       </c>
       <c r="K3" t="n">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="L3" t="n">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="M3" t="n">
-        <v>3.3843</v>
+        <v>3.2778</v>
       </c>
       <c r="N3" t="n">
-        <v>282</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>allu</t>
+          <t>KRIMZ</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.635</v>
+        <v>3.9105</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6623</v>
+        <v>0.7125</v>
       </c>
       <c r="D4" t="n">
-        <v>1.0043</v>
+        <v>1.1274</v>
       </c>
       <c r="E4" t="n">
-        <v>3.635</v>
+        <v>3.9105</v>
       </c>
       <c r="F4" t="n">
-        <v>2.0196</v>
+        <v>4.1605</v>
       </c>
       <c r="G4" t="n">
-        <v>1.6154</v>
+        <v>-0.25</v>
       </c>
       <c r="H4" t="n">
-        <v>2.0196</v>
+        <v>9.172700000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>1.6369</v>
+        <v>4.7694</v>
       </c>
       <c r="J4" t="n">
-        <v>1.6154</v>
+        <v>-0.25</v>
       </c>
       <c r="K4" t="n">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="L4" t="n">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="M4" t="n">
-        <v>3.2523</v>
+        <v>4.5194</v>
       </c>
       <c r="N4" t="n">
-        <v>198</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>f0rest</t>
+          <t>GeT_RiGhT</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.3305</v>
+        <v>3.5759</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6068</v>
+        <v>0.6515</v>
       </c>
       <c r="D5" t="n">
-        <v>0.883</v>
+        <v>0.9762999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>3.3305</v>
+        <v>3.5759</v>
       </c>
       <c r="F5" t="n">
-        <v>2.3753</v>
+        <v>1.7565</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9552</v>
+        <v>1.8194</v>
       </c>
       <c r="H5" t="n">
-        <v>2.3753</v>
+        <v>1.7565</v>
       </c>
       <c r="I5" t="n">
-        <v>1.9253</v>
+        <v>0.9133</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9552</v>
+        <v>1.8194</v>
       </c>
       <c r="K5" t="n">
         <v>80</v>
@@ -667,7 +667,7 @@
         <v>118</v>
       </c>
       <c r="M5" t="n">
-        <v>2.8805</v>
+        <v>2.7327</v>
       </c>
       <c r="N5" t="n">
         <v>198</v>
@@ -676,35 +676,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GeT_RiGhT</t>
+          <t>f0rest</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.0912</v>
+        <v>3.5648</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5632</v>
+        <v>0.6495</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7876</v>
+        <v>0.9713000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>3.0912</v>
+        <v>3.5648</v>
       </c>
       <c r="F6" t="n">
-        <v>1.1153</v>
+        <v>2.7084</v>
       </c>
       <c r="G6" t="n">
-        <v>1.9759</v>
+        <v>0.8564000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>1.1153</v>
+        <v>4.0563</v>
       </c>
       <c r="I6" t="n">
-        <v>0.904</v>
+        <v>2.1091</v>
       </c>
       <c r="J6" t="n">
-        <v>1.9759</v>
+        <v>0.8564000000000001</v>
       </c>
       <c r="K6" t="n">
         <v>80</v>
@@ -713,7 +713,7 @@
         <v>118</v>
       </c>
       <c r="M6" t="n">
-        <v>2.8799</v>
+        <v>2.9655</v>
       </c>
       <c r="N6" t="n">
         <v>198</v>
@@ -726,31 +726,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.1044</v>
+        <v>2.2144</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2012</v>
+        <v>0.4035</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0039</v>
+        <v>0.3617</v>
       </c>
       <c r="E7" t="n">
-        <v>1.1044</v>
+        <v>2.2144</v>
       </c>
       <c r="F7" t="n">
-        <v>1.8778</v>
+        <v>2.7994</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.7734</v>
+        <v>-0.585</v>
       </c>
       <c r="H7" t="n">
-        <v>1.8778</v>
+        <v>4.3769</v>
       </c>
       <c r="I7" t="n">
-        <v>1.522</v>
+        <v>2.2758</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.7734</v>
+        <v>-0.585</v>
       </c>
       <c r="K7" t="n">
         <v>143</v>
@@ -759,7 +759,7 @@
         <v>40</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7486</v>
+        <v>1.6908</v>
       </c>
       <c r="N7" t="n">
         <v>183</v>
@@ -768,173 +768,173 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Xyp9x</t>
+          <t>AcilioN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3437</v>
+        <v>1.2571</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0626</v>
+        <v>0.2291</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.307</v>
+        <v>-0.07049999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3437</v>
+        <v>1.2571</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5825</v>
+        <v>2.1115</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.2388</v>
+        <v>-0.8544</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5825</v>
+        <v>2.1115</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4721</v>
+        <v>1.0979</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.2388</v>
+        <v>-0.8544</v>
       </c>
       <c r="K8" t="n">
-        <v>72</v>
+        <v>143</v>
       </c>
       <c r="L8" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2333</v>
+        <v>0.2435</v>
       </c>
       <c r="N8" t="n">
-        <v>125</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AcilioN</t>
+          <t>Xyp9x</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.3153</v>
+        <v>0.6732</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0574</v>
+        <v>0.1227</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.3183</v>
+        <v>-0.3341</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3153</v>
+        <v>0.6732</v>
       </c>
       <c r="F9" t="n">
-        <v>1.3153</v>
+        <v>0.7718</v>
       </c>
       <c r="G9" t="n">
-        <v>-1</v>
+        <v>-0.09859999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>1.3153</v>
+        <v>0.7718</v>
       </c>
       <c r="I9" t="n">
-        <v>1.0661</v>
+        <v>0.4013</v>
       </c>
       <c r="J9" t="n">
-        <v>-1</v>
+        <v>-0.09859999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>143</v>
+        <v>72</v>
       </c>
       <c r="L9" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="M9" t="n">
-        <v>0.06610000000000005</v>
+        <v>0.3027</v>
       </c>
       <c r="N9" t="n">
-        <v>183</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Xizt</t>
+          <t>flusha</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2884</v>
+        <v>0.4997</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0525</v>
+        <v>0.091</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.329</v>
+        <v>-0.4124</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2884</v>
+        <v>0.4997</v>
       </c>
       <c r="F10" t="n">
-        <v>-1.0836</v>
+        <v>0.5193</v>
       </c>
       <c r="G10" t="n">
-        <v>1.372</v>
+        <v>-0.0196</v>
       </c>
       <c r="H10" t="n">
-        <v>-1.0836</v>
+        <v>0.5193</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.8783</v>
+        <v>0.27</v>
       </c>
       <c r="J10" t="n">
-        <v>1.372</v>
+        <v>-0.0196</v>
       </c>
       <c r="K10" t="n">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="L10" t="n">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="M10" t="n">
-        <v>0.4937000000000001</v>
+        <v>0.2504</v>
       </c>
       <c r="N10" t="n">
-        <v>198</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dennis</t>
+          <t>JW</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2664</v>
+        <v>0.4333</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0485</v>
+        <v>0.0789</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.3378</v>
+        <v>-0.4424</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2664</v>
+        <v>0.4333</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.838</v>
+        <v>-0.6487000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>1.1044</v>
+        <v>1.082</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.838</v>
+        <v>-0.6487000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.6792</v>
+        <v>-0.3373</v>
       </c>
       <c r="J11" t="n">
-        <v>1.1044</v>
+        <v>1.082</v>
       </c>
       <c r="K11" t="n">
         <v>151</v>
@@ -943,7 +943,7 @@
         <v>131</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4252</v>
+        <v>0.7447000000000001</v>
       </c>
       <c r="N11" t="n">
         <v>282</v>
@@ -952,139 +952,139 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dupreeh</t>
+          <t>dennis</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0068</v>
+        <v>0.4126</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0012</v>
+        <v>0.0752</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.4412</v>
+        <v>-0.4517</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0068</v>
+        <v>0.4126</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.0307</v>
+        <v>-0.6197</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0375</v>
+        <v>1.0323</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.0307</v>
+        <v>-0.6197</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.0249</v>
+        <v>-0.3222</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0375</v>
+        <v>1.0323</v>
       </c>
       <c r="K12" t="n">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="L12" t="n">
-        <v>53</v>
+        <v>131</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0126</v>
+        <v>0.7101</v>
       </c>
       <c r="N12" t="n">
-        <v>125</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>flusha</t>
+          <t>dupreeh</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.0732</v>
+        <v>0.2348</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.0133</v>
+        <v>0.0428</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.4731</v>
+        <v>-0.532</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.0732</v>
+        <v>0.2348</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0584</v>
+        <v>0.0323</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0148</v>
+        <v>0.2025</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0584</v>
+        <v>0.0323</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.0473</v>
+        <v>0.0168</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.0148</v>
+        <v>0.2025</v>
       </c>
       <c r="K13" t="n">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="L13" t="n">
-        <v>131</v>
+        <v>53</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.0621</v>
+        <v>0.2193</v>
       </c>
       <c r="N13" t="n">
-        <v>282</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>JW</t>
+          <t>Xizt</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.2041</v>
+        <v>0.0154</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.0372</v>
+        <v>0.0028</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.5252</v>
+        <v>-0.6311</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2041</v>
+        <v>0.0154</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.0061</v>
+        <v>-1.1905</v>
       </c>
       <c r="G14" t="n">
-        <v>0.802</v>
+        <v>1.2059</v>
       </c>
       <c r="H14" t="n">
-        <v>-1.0061</v>
+        <v>-1.1905</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.8155</v>
+        <v>-0.619</v>
       </c>
       <c r="J14" t="n">
-        <v>0.802</v>
+        <v>1.2059</v>
       </c>
       <c r="K14" t="n">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="L14" t="n">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.01349999999999996</v>
+        <v>0.5869</v>
       </c>
       <c r="N14" t="n">
-        <v>282</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15">
@@ -1094,31 +1094,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.6986</v>
+        <v>-0.3853</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.1273</v>
+        <v>-0.0702</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.7222</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.6986</v>
+        <v>-0.3853</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.8809</v>
+        <v>-0.6149</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1823</v>
+        <v>0.2296</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.8809</v>
+        <v>-0.6149</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.714</v>
+        <v>-0.3197</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1823</v>
+        <v>0.2296</v>
       </c>
       <c r="K15" t="n">
         <v>72</v>
@@ -1127,7 +1127,7 @@
         <v>53</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.5317</v>
+        <v>-0.09009999999999999</v>
       </c>
       <c r="N15" t="n">
         <v>125</v>
@@ -1136,35 +1136,35 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cadiaN</t>
+          <t>Magisk</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-1.0369</v>
+        <v>-0.3872</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.1889</v>
+        <v>-0.0706</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.857</v>
+        <v>-0.8128</v>
       </c>
       <c r="E16" t="n">
-        <v>-1.0369</v>
+        <v>-0.3872</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.7385</v>
+        <v>0.522</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.2984</v>
+        <v>-0.9092</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.7385</v>
+        <v>0.522</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.5986</v>
+        <v>0.2714</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.2984</v>
+        <v>-0.9092</v>
       </c>
       <c r="K16" t="n">
         <v>143</v>
@@ -1173,7 +1173,7 @@
         <v>40</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.897</v>
+        <v>-0.6378</v>
       </c>
       <c r="N16" t="n">
         <v>183</v>
@@ -1182,35 +1182,35 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Magisk</t>
+          <t>cadiaN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-1.2381</v>
+        <v>-0.7385</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.2256</v>
+        <v>-0.1346</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.9372</v>
+        <v>-0.9714</v>
       </c>
       <c r="E17" t="n">
-        <v>-1.2381</v>
+        <v>-0.7385</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.2381</v>
+        <v>-0.4631</v>
       </c>
       <c r="G17" t="n">
-        <v>-1</v>
+        <v>-0.2754</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.2381</v>
+        <v>-0.4631</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.193</v>
+        <v>-0.2408</v>
       </c>
       <c r="J17" t="n">
-        <v>-1</v>
+        <v>-0.2754</v>
       </c>
       <c r="K17" t="n">
         <v>143</v>
@@ -1219,7 +1219,7 @@
         <v>40</v>
       </c>
       <c r="M17" t="n">
-        <v>-1.193</v>
+        <v>-0.5162</v>
       </c>
       <c r="N17" t="n">
         <v>183</v>
@@ -1228,81 +1228,81 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>friberg</t>
+          <t>cajunb</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-1.4578</v>
+        <v>-1.319</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.2656</v>
+        <v>-0.2403</v>
       </c>
       <c r="D18" t="n">
-        <v>-1.0247</v>
+        <v>-1.2335</v>
       </c>
       <c r="E18" t="n">
-        <v>-1.4578</v>
+        <v>-1.319</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.6245</v>
+        <v>-1.0076</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1667</v>
+        <v>-0.3114</v>
       </c>
       <c r="H18" t="n">
-        <v>-1.6245</v>
+        <v>-1.0076</v>
       </c>
       <c r="I18" t="n">
-        <v>-1.3167</v>
+        <v>-0.5239</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1667</v>
+        <v>-0.3114</v>
       </c>
       <c r="K18" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="L18" t="n">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="M18" t="n">
-        <v>-1.15</v>
+        <v>-0.8353</v>
       </c>
       <c r="N18" t="n">
-        <v>198</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cajunb</t>
+          <t>karrigan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-1.5984</v>
+        <v>-1.5251</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.2912</v>
+        <v>-0.2779</v>
       </c>
       <c r="D19" t="n">
-        <v>-1.0807</v>
+        <v>-1.3265</v>
       </c>
       <c r="E19" t="n">
-        <v>-1.5984</v>
+        <v>-1.5251</v>
       </c>
       <c r="F19" t="n">
-        <v>-1.0709</v>
+        <v>-1.0366</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.5275</v>
+        <v>-0.4885</v>
       </c>
       <c r="H19" t="n">
-        <v>-1.0709</v>
+        <v>-1.0366</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.868</v>
+        <v>-0.539</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.5275</v>
+        <v>-0.4885</v>
       </c>
       <c r="K19" t="n">
         <v>72</v>
@@ -1311,7 +1311,7 @@
         <v>53</v>
       </c>
       <c r="M19" t="n">
-        <v>-1.3955</v>
+        <v>-1.0275</v>
       </c>
       <c r="N19" t="n">
         <v>125</v>
@@ -1320,47 +1320,47 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>karrigan</t>
+          <t>friberg</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-1.8674</v>
+        <v>-1.8139</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.3403</v>
+        <v>-0.3305</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.1879</v>
+        <v>-1.4569</v>
       </c>
       <c r="E20" t="n">
-        <v>-1.8674</v>
+        <v>-1.8139</v>
       </c>
       <c r="F20" t="n">
-        <v>-1.1617</v>
+        <v>-2.2708</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.7057</v>
+        <v>0.4569</v>
       </c>
       <c r="H20" t="n">
-        <v>-1.1617</v>
+        <v>-2.2708</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.9416</v>
+        <v>-1.1807</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.7057</v>
+        <v>0.4569</v>
       </c>
       <c r="K20" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L20" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="M20" t="n">
-        <v>-1.6473</v>
+        <v>-0.7238000000000001</v>
       </c>
       <c r="N20" t="n">
-        <v>125</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21">
@@ -1370,31 +1370,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-3.1925</v>
+        <v>-2.9582</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.5817</v>
+        <v>-0.539</v>
       </c>
       <c r="D21" t="n">
-        <v>-1.7158</v>
+        <v>-1.9735</v>
       </c>
       <c r="E21" t="n">
-        <v>-3.1925</v>
+        <v>-2.9582</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.1925</v>
+        <v>-2.196</v>
       </c>
       <c r="G21" t="n">
-        <v>-1</v>
+        <v>-0.7622</v>
       </c>
       <c r="H21" t="n">
-        <v>-2.1925</v>
+        <v>-2.196</v>
       </c>
       <c r="I21" t="n">
-        <v>-1.7771</v>
+        <v>-1.1418</v>
       </c>
       <c r="J21" t="n">
-        <v>-1</v>
+        <v>-0.7622</v>
       </c>
       <c r="K21" t="n">
         <v>143</v>
@@ -1403,7 +1403,7 @@
         <v>40</v>
       </c>
       <c r="M21" t="n">
-        <v>-2.7771</v>
+        <v>-1.904</v>
       </c>
       <c r="N21" t="n">
         <v>183</v>
@@ -1509,10 +1509,10 @@
         <v>1.14</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3989</v>
+        <v>0.4503</v>
       </c>
       <c r="J2" t="n">
-        <v>9.9725</v>
+        <v>11.2575</v>
       </c>
     </row>
     <row r="3">
@@ -1549,10 +1549,10 @@
         <v>0.74</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.3615</v>
+        <v>-0.265</v>
       </c>
       <c r="J3" t="n">
-        <v>-9.0375</v>
+        <v>-6.625</v>
       </c>
     </row>
     <row r="4">
@@ -1589,10 +1589,10 @@
         <v>0.67</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.4875</v>
+        <v>-0.3292</v>
       </c>
       <c r="J4" t="n">
-        <v>-12.1875</v>
+        <v>-8.23</v>
       </c>
     </row>
     <row r="5">
@@ -1629,10 +1629,10 @@
         <v>0.6</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.5885</v>
+        <v>-0.3947</v>
       </c>
       <c r="J5" t="n">
-        <v>-14.7125</v>
+        <v>-9.8675</v>
       </c>
     </row>
     <row r="6">
@@ -1669,10 +1669,10 @@
         <v>0.52</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.695</v>
+        <v>-0.4694</v>
       </c>
       <c r="J6" t="n">
-        <v>-17.375</v>
+        <v>-11.735</v>
       </c>
     </row>
     <row r="7">
@@ -1709,10 +1709,10 @@
         <v>1.54</v>
       </c>
       <c r="I7" t="n">
-        <v>1.2782</v>
+        <v>1.1806</v>
       </c>
       <c r="J7" t="n">
-        <v>31.955</v>
+        <v>29.515</v>
       </c>
     </row>
     <row r="8">
@@ -1749,10 +1749,10 @@
         <v>1.32</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8105</v>
+        <v>0.8266</v>
       </c>
       <c r="J8" t="n">
-        <v>20.2625</v>
+        <v>20.665</v>
       </c>
     </row>
     <row r="9">
@@ -1789,10 +1789,10 @@
         <v>1.23</v>
       </c>
       <c r="I9" t="n">
-        <v>0.5647</v>
+        <v>0.6236</v>
       </c>
       <c r="J9" t="n">
-        <v>14.1175</v>
+        <v>15.59</v>
       </c>
     </row>
     <row r="10">
@@ -1829,10 +1829,10 @@
         <v>1.08</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1568</v>
+        <v>0.2333</v>
       </c>
       <c r="J10" t="n">
-        <v>3.92</v>
+        <v>5.8325</v>
       </c>
     </row>
     <row r="11">
@@ -1869,10 +1869,10 @@
         <v>1.07</v>
       </c>
       <c r="I11" t="n">
-        <v>0.127</v>
+        <v>0.2033</v>
       </c>
       <c r="J11" t="n">
-        <v>3.175</v>
+        <v>5.0825</v>
       </c>
     </row>
     <row r="12">
@@ -1909,10 +1909,10 @@
         <v>1.44</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6432</v>
+        <v>0.5652</v>
       </c>
       <c r="J12" t="n">
-        <v>16.08</v>
+        <v>14.13</v>
       </c>
     </row>
     <row r="13">
@@ -1949,10 +1949,10 @@
         <v>1.29</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4542</v>
+        <v>0.393</v>
       </c>
       <c r="J13" t="n">
-        <v>11.355</v>
+        <v>9.824999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -1989,10 +1989,10 @@
         <v>1.24</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3846</v>
+        <v>0.3335</v>
       </c>
       <c r="J14" t="n">
-        <v>9.615</v>
+        <v>8.3375</v>
       </c>
     </row>
     <row r="15">
@@ -2029,10 +2029,10 @@
         <v>1.06</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0766</v>
+        <v>0.0973</v>
       </c>
       <c r="J15" t="n">
-        <v>1.915</v>
+        <v>2.4325</v>
       </c>
     </row>
     <row r="16">
@@ -2069,10 +2069,10 @@
         <v>0.78</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.4411</v>
+        <v>-0.276</v>
       </c>
       <c r="J16" t="n">
-        <v>-11.0275</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="17">
@@ -2109,10 +2109,10 @@
         <v>1.34</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6586</v>
+        <v>0.6261</v>
       </c>
       <c r="J17" t="n">
-        <v>16.465</v>
+        <v>15.6525</v>
       </c>
     </row>
     <row r="18">
@@ -2149,10 +2149,10 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1061</v>
+        <v>0.0527</v>
       </c>
       <c r="J18" t="n">
-        <v>2.6525</v>
+        <v>1.3175</v>
       </c>
     </row>
     <row r="19">
@@ -2189,10 +2189,10 @@
         <v>0.62</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.5737</v>
+        <v>-0.3822</v>
       </c>
       <c r="J19" t="n">
-        <v>-14.3425</v>
+        <v>-9.555</v>
       </c>
     </row>
     <row r="20">
@@ -2229,10 +2229,10 @@
         <v>0.59</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.614</v>
+        <v>-0.4102</v>
       </c>
       <c r="J20" t="n">
-        <v>-15.35</v>
+        <v>-10.255</v>
       </c>
     </row>
     <row r="21">
@@ -2269,10 +2269,10 @@
         <v>0.32</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.9427</v>
+        <v>-0.6588000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>-23.5675</v>
+        <v>-16.47</v>
       </c>
     </row>
     <row r="22">
@@ -2309,10 +2309,10 @@
         <v>1.26</v>
       </c>
       <c r="I22" t="n">
-        <v>0.4881</v>
+        <v>0.5706</v>
       </c>
       <c r="J22" t="n">
-        <v>13.6668</v>
+        <v>15.9768</v>
       </c>
     </row>
     <row r="23">
@@ -2349,10 +2349,10 @@
         <v>1.03</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1192</v>
+        <v>0.105</v>
       </c>
       <c r="J23" t="n">
-        <v>3.3376</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="24">
@@ -2389,10 +2389,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.1213</v>
+        <v>-0.0829</v>
       </c>
       <c r="J24" t="n">
-        <v>-3.3964</v>
+        <v>-2.3212</v>
       </c>
     </row>
     <row r="25">
@@ -2429,10 +2429,10 @@
         <v>0.88</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.2409</v>
+        <v>-0.1494</v>
       </c>
       <c r="J25" t="n">
-        <v>-6.7452</v>
+        <v>-4.1832</v>
       </c>
     </row>
     <row r="26">
@@ -2469,10 +2469,10 @@
         <v>0.59</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.6489</v>
+        <v>-0.4319</v>
       </c>
       <c r="J26" t="n">
-        <v>-18.1692</v>
+        <v>-12.0932</v>
       </c>
     </row>
     <row r="27">
@@ -2509,10 +2509,10 @@
         <v>1.44</v>
       </c>
       <c r="I27" t="n">
-        <v>1.1854</v>
+        <v>1.1096</v>
       </c>
       <c r="J27" t="n">
-        <v>33.1912</v>
+        <v>31.0688</v>
       </c>
     </row>
     <row r="28">
@@ -2549,10 +2549,10 @@
         <v>1.18</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5933</v>
+        <v>0.5533</v>
       </c>
       <c r="J28" t="n">
-        <v>16.6124</v>
+        <v>15.4924</v>
       </c>
     </row>
     <row r="29">
@@ -2589,10 +2589,10 @@
         <v>0.98</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.1477</v>
+        <v>-0.1025</v>
       </c>
       <c r="J29" t="n">
-        <v>-4.1356</v>
+        <v>-2.87</v>
       </c>
     </row>
     <row r="30">
@@ -2629,10 +2629,10 @@
         <v>0.96</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.2246</v>
+        <v>-0.1742</v>
       </c>
       <c r="J30" t="n">
-        <v>-6.2888</v>
+        <v>-4.8776</v>
       </c>
     </row>
     <row r="31">
@@ -2669,10 +2669,10 @@
         <v>0.63</v>
       </c>
       <c r="I31" t="n">
-        <v>-1.0695</v>
+        <v>-1.054</v>
       </c>
       <c r="J31" t="n">
-        <v>-29.946</v>
+        <v>-29.512</v>
       </c>
     </row>
     <row r="32">
@@ -2709,10 +2709,10 @@
         <v>1.78</v>
       </c>
       <c r="I32" t="n">
-        <v>1.0157</v>
+        <v>0.9325</v>
       </c>
       <c r="J32" t="n">
-        <v>28.4396</v>
+        <v>26.11</v>
       </c>
     </row>
     <row r="33">
@@ -2749,10 +2749,10 @@
         <v>1.19</v>
       </c>
       <c r="I33" t="n">
-        <v>0.3098</v>
+        <v>0.2729</v>
       </c>
       <c r="J33" t="n">
-        <v>8.6744</v>
+        <v>7.6412</v>
       </c>
     </row>
     <row r="34">
@@ -2789,10 +2789,10 @@
         <v>1.04</v>
       </c>
       <c r="I34" t="n">
-        <v>0.0388</v>
+        <v>0.065</v>
       </c>
       <c r="J34" t="n">
-        <v>1.0864</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="35">
@@ -2829,10 +2829,10 @@
         <v>1.03</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0183</v>
+        <v>0.0475</v>
       </c>
       <c r="J35" t="n">
-        <v>0.5124</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="36">
@@ -2869,10 +2869,10 @@
         <v>0.76</v>
       </c>
       <c r="I36" t="n">
-        <v>-0.4674</v>
+        <v>-0.2953</v>
       </c>
       <c r="J36" t="n">
-        <v>-13.0872</v>
+        <v>-8.2684</v>
       </c>
     </row>
     <row r="37">
@@ -2909,10 +2909,10 @@
         <v>1.44</v>
       </c>
       <c r="I37" t="n">
-        <v>0.7212</v>
+        <v>0.6849</v>
       </c>
       <c r="J37" t="n">
-        <v>20.1936</v>
+        <v>19.1772</v>
       </c>
     </row>
     <row r="38">
@@ -2949,10 +2949,10 @@
         <v>1.14</v>
       </c>
       <c r="I38" t="n">
-        <v>0.3221</v>
+        <v>0.2686</v>
       </c>
       <c r="J38" t="n">
-        <v>9.018800000000001</v>
+        <v>7.5208</v>
       </c>
     </row>
     <row r="39">
@@ -2989,10 +2989,10 @@
         <v>0.86</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.2678</v>
+        <v>-0.1685</v>
       </c>
       <c r="J39" t="n">
-        <v>-7.4984</v>
+        <v>-4.718</v>
       </c>
     </row>
     <row r="40">
@@ -3029,10 +3029,10 @@
         <v>0.85</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.2844</v>
+        <v>-0.1788</v>
       </c>
       <c r="J40" t="n">
-        <v>-7.9632</v>
+        <v>-5.0064</v>
       </c>
     </row>
     <row r="41">
@@ -3069,10 +3069,10 @@
         <v>0.32</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.9568</v>
+        <v>-0.6715</v>
       </c>
       <c r="J41" t="n">
-        <v>-26.7904</v>
+        <v>-18.802</v>
       </c>
     </row>
     <row r="42">
@@ -3109,10 +3109,10 @@
         <v>1.06</v>
       </c>
       <c r="I42" t="n">
-        <v>0.2513</v>
+        <v>0.2499</v>
       </c>
       <c r="J42" t="n">
-        <v>5.2773</v>
+        <v>5.2479</v>
       </c>
     </row>
     <row r="43">
@@ -3149,10 +3149,10 @@
         <v>0.91</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.0868</v>
+        <v>-0.0922</v>
       </c>
       <c r="J43" t="n">
-        <v>-1.8228</v>
+        <v>-1.9362</v>
       </c>
     </row>
     <row r="44">
@@ -3189,10 +3189,10 @@
         <v>0.78</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.3096</v>
+        <v>-0.2311</v>
       </c>
       <c r="J44" t="n">
-        <v>-6.5016</v>
+        <v>-4.8531</v>
       </c>
     </row>
     <row r="45">
@@ -3229,10 +3229,10 @@
         <v>0.62</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.5706</v>
+        <v>-0.3806</v>
       </c>
       <c r="J45" t="n">
-        <v>-11.9826</v>
+        <v>-7.9926</v>
       </c>
     </row>
     <row r="46">
@@ -3269,10 +3269,10 @@
         <v>0.45</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.7889</v>
+        <v>-0.5387</v>
       </c>
       <c r="J46" t="n">
-        <v>-16.5669</v>
+        <v>-11.3127</v>
       </c>
     </row>
     <row r="47">
@@ -3309,10 +3309,10 @@
         <v>1.47</v>
       </c>
       <c r="I47" t="n">
-        <v>1.1706</v>
+        <v>1.1072</v>
       </c>
       <c r="J47" t="n">
-        <v>24.5826</v>
+        <v>23.2512</v>
       </c>
     </row>
     <row r="48">
@@ -3349,10 +3349,10 @@
         <v>1.4</v>
       </c>
       <c r="I48" t="n">
-        <v>1.0249</v>
+        <v>1.0101</v>
       </c>
       <c r="J48" t="n">
-        <v>21.5229</v>
+        <v>21.2121</v>
       </c>
     </row>
     <row r="49">
@@ -3389,10 +3389,10 @@
         <v>1.19</v>
       </c>
       <c r="I49" t="n">
-        <v>0.519</v>
+        <v>0.5387</v>
       </c>
       <c r="J49" t="n">
-        <v>10.899</v>
+        <v>11.3127</v>
       </c>
     </row>
     <row r="50">
@@ -3429,10 +3429,10 @@
         <v>0.95</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.3224</v>
+        <v>-0.2459</v>
       </c>
       <c r="J50" t="n">
-        <v>-6.7704</v>
+        <v>-5.1639</v>
       </c>
     </row>
     <row r="51">
@@ -3469,10 +3469,10 @@
         <v>0.9</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.4707</v>
+        <v>-0.3989</v>
       </c>
       <c r="J51" t="n">
-        <v>-9.8847</v>
+        <v>-8.376899999999999</v>
       </c>
     </row>
     <row r="52">
@@ -3509,10 +3509,10 @@
         <v>0.85</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.0961</v>
+        <v>-0.1055</v>
       </c>
       <c r="J52" t="n">
-        <v>-2.1142</v>
+        <v>-2.321</v>
       </c>
     </row>
     <row r="53">
@@ -3549,10 +3549,10 @@
         <v>0.78</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.2071</v>
+        <v>-0.1872</v>
       </c>
       <c r="J53" t="n">
-        <v>-4.5562</v>
+        <v>-4.1184</v>
       </c>
     </row>
     <row r="54">
@@ -3589,10 +3589,10 @@
         <v>0.47</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.7137</v>
+        <v>-0.4897</v>
       </c>
       <c r="J54" t="n">
-        <v>-15.7014</v>
+        <v>-10.7734</v>
       </c>
     </row>
     <row r="55">
@@ -3629,10 +3629,10 @@
         <v>0.47</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.7137</v>
+        <v>-0.4897</v>
       </c>
       <c r="J55" t="n">
-        <v>-15.7014</v>
+        <v>-10.7734</v>
       </c>
     </row>
     <row r="56">
@@ -3669,10 +3669,10 @@
         <v>0.34</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.8871</v>
+        <v>-0.6145</v>
       </c>
       <c r="J56" t="n">
-        <v>-19.5162</v>
+        <v>-13.519</v>
       </c>
     </row>
     <row r="57">
@@ -3709,10 +3709,10 @@
         <v>1.84</v>
       </c>
       <c r="I57" t="n">
-        <v>1.7527</v>
+        <v>1.4997</v>
       </c>
       <c r="J57" t="n">
-        <v>38.5594</v>
+        <v>32.9934</v>
       </c>
     </row>
     <row r="58">
@@ -3749,10 +3749,10 @@
         <v>1.64</v>
       </c>
       <c r="I58" t="n">
-        <v>1.3905</v>
+        <v>1.2675</v>
       </c>
       <c r="J58" t="n">
-        <v>30.591</v>
+        <v>27.885</v>
       </c>
     </row>
     <row r="59">
@@ -3789,10 +3789,10 @@
         <v>1.31</v>
       </c>
       <c r="I59" t="n">
-        <v>0.6623</v>
+        <v>0.7738</v>
       </c>
       <c r="J59" t="n">
-        <v>14.5706</v>
+        <v>17.0236</v>
       </c>
     </row>
     <row r="60">
@@ -3829,10 +3829,10 @@
         <v>1.26</v>
       </c>
       <c r="I60" t="n">
-        <v>0.5486</v>
+        <v>0.6592</v>
       </c>
       <c r="J60" t="n">
-        <v>12.0692</v>
+        <v>14.5024</v>
       </c>
     </row>
     <row r="61">
@@ -3869,10 +3869,10 @@
         <v>1.07</v>
       </c>
       <c r="I61" t="n">
-        <v>0.0728</v>
+        <v>0.1635</v>
       </c>
       <c r="J61" t="n">
-        <v>1.6016</v>
+        <v>3.597</v>
       </c>
     </row>
     <row r="62">
@@ -3909,10 +3909,10 @@
         <v>1.4</v>
       </c>
       <c r="I62" t="n">
-        <v>1.052</v>
+        <v>1.0249</v>
       </c>
       <c r="J62" t="n">
-        <v>23.144</v>
+        <v>22.5478</v>
       </c>
     </row>
     <row r="63">
@@ -3949,10 +3949,10 @@
         <v>1.36</v>
       </c>
       <c r="I63" t="n">
-        <v>0.966</v>
+        <v>0.9524</v>
       </c>
       <c r="J63" t="n">
-        <v>21.252</v>
+        <v>20.9528</v>
       </c>
     </row>
     <row r="64">
@@ -3989,10 +3989,10 @@
         <v>1.11</v>
       </c>
       <c r="I64" t="n">
-        <v>0.3099</v>
+        <v>0.3455</v>
       </c>
       <c r="J64" t="n">
-        <v>6.8178</v>
+        <v>7.601</v>
       </c>
     </row>
     <row r="65">
@@ -4029,10 +4029,10 @@
         <v>0.97</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.2343</v>
+        <v>-0.1639</v>
       </c>
       <c r="J65" t="n">
-        <v>-5.1546</v>
+        <v>-3.6058</v>
       </c>
     </row>
     <row r="66">
@@ -4069,10 +4069,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.6873</v>
+        <v>-0.6317</v>
       </c>
       <c r="J66" t="n">
-        <v>-15.1206</v>
+        <v>-13.8974</v>
       </c>
     </row>
     <row r="67">
@@ -4109,10 +4109,10 @@
         <v>1.29</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5901999999999999</v>
+        <v>0.7171999999999999</v>
       </c>
       <c r="J67" t="n">
-        <v>12.9844</v>
+        <v>15.7784</v>
       </c>
     </row>
     <row r="68">
@@ -4149,10 +4149,10 @@
         <v>0.77</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.3495</v>
+        <v>-0.2418</v>
       </c>
       <c r="J68" t="n">
-        <v>-7.689</v>
+        <v>-5.3196</v>
       </c>
     </row>
     <row r="69">
@@ -4189,10 +4189,10 @@
         <v>0.75</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.3846</v>
+        <v>-0.2606</v>
       </c>
       <c r="J69" t="n">
-        <v>-8.4612</v>
+        <v>-5.7332</v>
       </c>
     </row>
     <row r="70">
@@ -4229,10 +4229,10 @@
         <v>0.73</v>
       </c>
       <c r="I70" t="n">
-        <v>-0.417</v>
+        <v>-0.2795</v>
       </c>
       <c r="J70" t="n">
-        <v>-9.173999999999999</v>
+        <v>-6.149</v>
       </c>
     </row>
     <row r="71">
@@ -4269,10 +4269,10 @@
         <v>0.37</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.8864</v>
+        <v>-0.6142</v>
       </c>
       <c r="J71" t="n">
-        <v>-19.5008</v>
+        <v>-13.5124</v>
       </c>
     </row>
     <row r="72">
@@ -4309,10 +4309,10 @@
         <v>1.13</v>
       </c>
       <c r="I72" t="n">
-        <v>0.2916</v>
+        <v>0.2429</v>
       </c>
       <c r="J72" t="n">
-        <v>8.747999999999999</v>
+        <v>7.287</v>
       </c>
     </row>
     <row r="73">
@@ -4349,10 +4349,10 @@
         <v>1.09</v>
       </c>
       <c r="I73" t="n">
-        <v>0.2253</v>
+        <v>0.1804</v>
       </c>
       <c r="J73" t="n">
-        <v>6.759</v>
+        <v>5.412</v>
       </c>
     </row>
     <row r="74">
@@ -4389,10 +4389,10 @@
         <v>0.97</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.0634</v>
+        <v>-0.0473</v>
       </c>
       <c r="J74" t="n">
-        <v>-1.902</v>
+        <v>-1.419</v>
       </c>
     </row>
     <row r="75">
@@ -4429,10 +4429,10 @@
         <v>0.89</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.2321</v>
+        <v>-0.141</v>
       </c>
       <c r="J75" t="n">
-        <v>-6.963</v>
+        <v>-4.23</v>
       </c>
     </row>
     <row r="76">
@@ -4469,10 +4469,10 @@
         <v>0.73</v>
       </c>
       <c r="I76" t="n">
-        <v>-0.4728</v>
+        <v>-0.3032</v>
       </c>
       <c r="J76" t="n">
-        <v>-14.184</v>
+        <v>-9.096</v>
       </c>
     </row>
     <row r="77">
@@ -4509,10 +4509,10 @@
         <v>1.74</v>
       </c>
       <c r="I77" t="n">
-        <v>1.0021</v>
+        <v>0.9217</v>
       </c>
       <c r="J77" t="n">
-        <v>30.063</v>
+        <v>27.651</v>
       </c>
     </row>
     <row r="78">
@@ -4549,10 +4549,10 @@
         <v>1.07</v>
       </c>
       <c r="I78" t="n">
-        <v>0.1364</v>
+        <v>0.1224</v>
       </c>
       <c r="J78" t="n">
-        <v>4.092</v>
+        <v>3.672</v>
       </c>
     </row>
     <row r="79">
@@ -4589,10 +4589,10 @@
         <v>0.92</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.2135</v>
+        <v>-0.1192</v>
       </c>
       <c r="J79" t="n">
-        <v>-6.405</v>
+        <v>-3.576</v>
       </c>
     </row>
     <row r="80">
@@ -4629,10 +4629,10 @@
         <v>0.89</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.2636</v>
+        <v>-0.153</v>
       </c>
       <c r="J80" t="n">
-        <v>-7.908</v>
+        <v>-4.59</v>
       </c>
     </row>
     <row r="81">
@@ -4669,10 +4669,10 @@
         <v>0.73</v>
       </c>
       <c r="I81" t="n">
-        <v>-0.4931</v>
+        <v>-0.3152</v>
       </c>
       <c r="J81" t="n">
-        <v>-14.793</v>
+        <v>-9.456</v>
       </c>
     </row>
     <row r="82">
@@ -4709,10 +4709,10 @@
         <v>1.61</v>
       </c>
       <c r="I82" t="n">
-        <v>1.4641</v>
+        <v>1.2977</v>
       </c>
       <c r="J82" t="n">
-        <v>40.9948</v>
+        <v>36.3356</v>
       </c>
     </row>
     <row r="83">
@@ -4749,10 +4749,10 @@
         <v>1.31</v>
       </c>
       <c r="I83" t="n">
-        <v>0.8467</v>
+        <v>0.8343</v>
       </c>
       <c r="J83" t="n">
-        <v>23.7076</v>
+        <v>23.3604</v>
       </c>
     </row>
     <row r="84">
@@ -4789,10 +4789,10 @@
         <v>1.14</v>
       </c>
       <c r="I84" t="n">
-        <v>0.3941</v>
+        <v>0.4216</v>
       </c>
       <c r="J84" t="n">
-        <v>11.0348</v>
+        <v>11.8048</v>
       </c>
     </row>
     <row r="85">
@@ -4829,10 +4829,10 @@
         <v>0.86</v>
       </c>
       <c r="I85" t="n">
-        <v>-0.5659999999999999</v>
+        <v>-0.5017</v>
       </c>
       <c r="J85" t="n">
-        <v>-15.848</v>
+        <v>-14.0476</v>
       </c>
     </row>
     <row r="86">
@@ -4869,10 +4869,10 @@
         <v>0.8</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.7154</v>
+        <v>-0.6613</v>
       </c>
       <c r="J86" t="n">
-        <v>-20.0312</v>
+        <v>-18.5164</v>
       </c>
     </row>
     <row r="87">
@@ -4909,10 +4909,10 @@
         <v>1.23</v>
       </c>
       <c r="I87" t="n">
-        <v>0.4848</v>
+        <v>0.5646</v>
       </c>
       <c r="J87" t="n">
-        <v>13.5744</v>
+        <v>15.8088</v>
       </c>
     </row>
     <row r="88">
@@ -4949,10 +4949,10 @@
         <v>0.95</v>
       </c>
       <c r="I88" t="n">
-        <v>-0.046</v>
+        <v>-0.0578</v>
       </c>
       <c r="J88" t="n">
-        <v>-1.288</v>
+        <v>-1.6184</v>
       </c>
     </row>
     <row r="89">
@@ -4989,10 +4989,10 @@
         <v>0.92</v>
       </c>
       <c r="I89" t="n">
-        <v>-0.1035</v>
+        <v>-0.0948</v>
       </c>
       <c r="J89" t="n">
-        <v>-2.898</v>
+        <v>-2.6544</v>
       </c>
     </row>
     <row r="90">
@@ -5029,10 +5029,10 @@
         <v>0.64</v>
       </c>
       <c r="I90" t="n">
-        <v>-0.5649</v>
+        <v>-0.3729</v>
       </c>
       <c r="J90" t="n">
-        <v>-15.8172</v>
+        <v>-10.4412</v>
       </c>
     </row>
     <row r="91">
@@ -5069,10 +5069,10 @@
         <v>0.46</v>
       </c>
       <c r="I91" t="n">
-        <v>-0.7895</v>
+        <v>-0.539</v>
       </c>
       <c r="J91" t="n">
-        <v>-22.106</v>
+        <v>-15.092</v>
       </c>
     </row>
     <row r="92">
@@ -5109,10 +5109,10 @@
         <v>1.84</v>
       </c>
       <c r="I92" t="n">
-        <v>1.7036</v>
+        <v>1.476</v>
       </c>
       <c r="J92" t="n">
-        <v>30.6648</v>
+        <v>26.568</v>
       </c>
     </row>
     <row r="93">
@@ -5149,10 +5149,10 @@
         <v>1.63</v>
       </c>
       <c r="I93" t="n">
-        <v>1.3152</v>
+        <v>1.2388</v>
       </c>
       <c r="J93" t="n">
-        <v>23.6736</v>
+        <v>22.2984</v>
       </c>
     </row>
     <row r="94">
@@ -5189,10 +5189,10 @@
         <v>1.51</v>
       </c>
       <c r="I94" t="n">
-        <v>1.0432</v>
+        <v>1.1024</v>
       </c>
       <c r="J94" t="n">
-        <v>18.7776</v>
+        <v>19.8432</v>
       </c>
     </row>
     <row r="95">
@@ -5229,10 +5229,10 @@
         <v>1.45</v>
       </c>
       <c r="I95" t="n">
-        <v>0.9152</v>
+        <v>1.0283</v>
       </c>
       <c r="J95" t="n">
-        <v>16.4736</v>
+        <v>18.5094</v>
       </c>
     </row>
     <row r="96">
@@ -5269,10 +5269,10 @@
         <v>1.3</v>
       </c>
       <c r="I96" t="n">
-        <v>0.5977</v>
+        <v>0.7271</v>
       </c>
       <c r="J96" t="n">
-        <v>10.7586</v>
+        <v>13.0878</v>
       </c>
     </row>
     <row r="97">
@@ -5309,10 +5309,10 @@
         <v>0.73</v>
       </c>
       <c r="I97" t="n">
-        <v>-0.2021</v>
+        <v>-0.1817</v>
       </c>
       <c r="J97" t="n">
-        <v>-3.6378</v>
+        <v>-3.2706</v>
       </c>
     </row>
     <row r="98">
@@ -5349,10 +5349,10 @@
         <v>0.73</v>
       </c>
       <c r="I98" t="n">
-        <v>-0.2021</v>
+        <v>-0.1817</v>
       </c>
       <c r="J98" t="n">
-        <v>-3.6378</v>
+        <v>-3.2706</v>
       </c>
     </row>
     <row r="99">
@@ -5389,10 +5389,10 @@
         <v>0.45</v>
       </c>
       <c r="I99" t="n">
-        <v>-0.6646</v>
+        <v>-0.4821</v>
       </c>
       <c r="J99" t="n">
-        <v>-11.9628</v>
+        <v>-8.6778</v>
       </c>
     </row>
     <row r="100">
@@ -5429,10 +5429,10 @@
         <v>0.23</v>
       </c>
       <c r="I100" t="n">
-        <v>-0.9987</v>
+        <v>-0.7010999999999999</v>
       </c>
       <c r="J100" t="n">
-        <v>-17.9766</v>
+        <v>-12.6198</v>
       </c>
     </row>
     <row r="101">
@@ -5469,10 +5469,10 @@
         <v>0.14</v>
       </c>
       <c r="I101" t="n">
-        <v>-1.115</v>
+        <v>-0.7961</v>
       </c>
       <c r="J101" t="n">
-        <v>-20.07</v>
+        <v>-14.3298</v>
       </c>
     </row>
     <row r="102">
@@ -5509,10 +5509,10 @@
         <v>1.1</v>
       </c>
       <c r="I102" t="n">
-        <v>0.3302</v>
+        <v>0.2719</v>
       </c>
       <c r="J102" t="n">
-        <v>8.255000000000001</v>
+        <v>6.7975</v>
       </c>
     </row>
     <row r="103">
@@ -5549,10 +5549,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="I103" t="n">
-        <v>-0.2462</v>
+        <v>-0.1984</v>
       </c>
       <c r="J103" t="n">
-        <v>-6.155</v>
+        <v>-4.96</v>
       </c>
     </row>
     <row r="104">
@@ -5589,10 +5589,10 @@
         <v>0.72</v>
       </c>
       <c r="I104" t="n">
-        <v>-0.4128</v>
+        <v>-0.284</v>
       </c>
       <c r="J104" t="n">
-        <v>-10.32</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="105">
@@ -5629,10 +5629,10 @@
         <v>0.7</v>
       </c>
       <c r="I105" t="n">
-        <v>-0.4457</v>
+        <v>-0.3026</v>
       </c>
       <c r="J105" t="n">
-        <v>-11.1425</v>
+        <v>-7.565</v>
       </c>
     </row>
     <row r="106">
@@ -5669,10 +5669,10 @@
         <v>0.39</v>
       </c>
       <c r="I106" t="n">
-        <v>-0.8574000000000001</v>
+        <v>-0.5913</v>
       </c>
       <c r="J106" t="n">
-        <v>-21.435</v>
+        <v>-14.7825</v>
       </c>
     </row>
     <row r="107">
@@ -5709,10 +5709,10 @@
         <v>1.42</v>
       </c>
       <c r="I107" t="n">
-        <v>0.6133999999999999</v>
+        <v>0.5387</v>
       </c>
       <c r="J107" t="n">
-        <v>15.335</v>
+        <v>13.4675</v>
       </c>
     </row>
     <row r="108">
@@ -5749,10 +5749,10 @@
         <v>1.3</v>
       </c>
       <c r="I108" t="n">
-        <v>0.4611</v>
+        <v>0.4017</v>
       </c>
       <c r="J108" t="n">
-        <v>11.5275</v>
+        <v>10.0425</v>
       </c>
     </row>
     <row r="109">
@@ -5789,10 +5789,10 @@
         <v>1.2</v>
       </c>
       <c r="I109" t="n">
-        <v>0.3155</v>
+        <v>0.283</v>
       </c>
       <c r="J109" t="n">
-        <v>7.8875</v>
+        <v>7.075</v>
       </c>
     </row>
     <row r="110">
@@ -5829,10 +5829,10 @@
         <v>1.04</v>
       </c>
       <c r="I110" t="n">
-        <v>0.0331</v>
+        <v>0.0622</v>
       </c>
       <c r="J110" t="n">
-        <v>0.8275</v>
+        <v>1.555</v>
       </c>
     </row>
     <row r="111">
@@ -5869,10 +5869,10 @@
         <v>0.95</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.1853</v>
+        <v>-0.0946</v>
       </c>
       <c r="J111" t="n">
-        <v>-4.6325</v>
+        <v>-2.365</v>
       </c>
     </row>
     <row r="112">
@@ -5909,10 +5909,10 @@
         <v>1.44</v>
       </c>
       <c r="I112" t="n">
-        <v>1.2095</v>
+        <v>1.1253</v>
       </c>
       <c r="J112" t="n">
-        <v>35.0755</v>
+        <v>32.6337</v>
       </c>
     </row>
     <row r="113">
@@ -5949,10 +5949,10 @@
         <v>0.99</v>
       </c>
       <c r="I113" t="n">
-        <v>-0.0654</v>
+        <v>-0.0527</v>
       </c>
       <c r="J113" t="n">
-        <v>-1.8966</v>
+        <v>-1.5283</v>
       </c>
     </row>
     <row r="114">
@@ -5989,10 +5989,10 @@
         <v>0.96</v>
       </c>
       <c r="I114" t="n">
-        <v>-0.1961</v>
+        <v>-0.1634</v>
       </c>
       <c r="J114" t="n">
-        <v>-5.6869</v>
+        <v>-4.7386</v>
       </c>
     </row>
     <row r="115">
@@ -6029,10 +6029,10 @@
         <v>0.86</v>
       </c>
       <c r="I115" t="n">
-        <v>-0.5086000000000001</v>
+        <v>-0.46</v>
       </c>
       <c r="J115" t="n">
-        <v>-14.7494</v>
+        <v>-13.34</v>
       </c>
     </row>
     <row r="116">
@@ -6069,10 +6069,10 @@
         <v>0.73</v>
       </c>
       <c r="I116" t="n">
-        <v>-0.8349</v>
+        <v>-0.7982</v>
       </c>
       <c r="J116" t="n">
-        <v>-24.2121</v>
+        <v>-23.1478</v>
       </c>
     </row>
     <row r="117">
@@ -6109,10 +6109,10 @@
         <v>1.18</v>
       </c>
       <c r="I117" t="n">
-        <v>0.3679</v>
+        <v>0.4142</v>
       </c>
       <c r="J117" t="n">
-        <v>10.6691</v>
+        <v>12.0118</v>
       </c>
     </row>
     <row r="118">
@@ -6149,10 +6149,10 @@
         <v>1.1</v>
       </c>
       <c r="I118" t="n">
-        <v>0.2424</v>
+        <v>0.2567</v>
       </c>
       <c r="J118" t="n">
-        <v>7.0296</v>
+        <v>7.4443</v>
       </c>
     </row>
     <row r="119">
@@ -6189,10 +6189,10 @@
         <v>1.01</v>
       </c>
       <c r="I119" t="n">
-        <v>0.0608</v>
+        <v>0.0443</v>
       </c>
       <c r="J119" t="n">
-        <v>1.7632</v>
+        <v>1.2847</v>
       </c>
     </row>
     <row r="120">
@@ -6229,10 +6229,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I120" t="n">
-        <v>-0.1383</v>
+        <v>-0.08450000000000001</v>
       </c>
       <c r="J120" t="n">
-        <v>-4.0107</v>
+        <v>-2.4505</v>
       </c>
     </row>
     <row r="121">
@@ -6269,10 +6269,10 @@
         <v>0.58</v>
       </c>
       <c r="I121" t="n">
-        <v>-0.6645</v>
+        <v>-0.4435</v>
       </c>
       <c r="J121" t="n">
-        <v>-19.2705</v>
+        <v>-12.8615</v>
       </c>
     </row>
     <row r="122">
@@ -6309,10 +6309,10 @@
         <v>1.21</v>
       </c>
       <c r="I122" t="n">
-        <v>0.6407</v>
+        <v>0.4982</v>
       </c>
       <c r="J122" t="n">
-        <v>17.2989</v>
+        <v>13.4514</v>
       </c>
     </row>
     <row r="123">
@@ -6349,10 +6349,10 @@
         <v>1.14</v>
       </c>
       <c r="I123" t="n">
-        <v>0.4534</v>
+        <v>0.3923</v>
       </c>
       <c r="J123" t="n">
-        <v>12.2418</v>
+        <v>10.5921</v>
       </c>
     </row>
     <row r="124">
@@ -6389,10 +6389,10 @@
         <v>1.13</v>
       </c>
       <c r="I124" t="n">
-        <v>0.4243</v>
+        <v>0.3766</v>
       </c>
       <c r="J124" t="n">
-        <v>11.4561</v>
+        <v>10.1682</v>
       </c>
     </row>
     <row r="125">
@@ -6429,10 +6429,10 @@
         <v>1.13</v>
       </c>
       <c r="I125" t="n">
-        <v>0.4243</v>
+        <v>0.3766</v>
       </c>
       <c r="J125" t="n">
-        <v>11.4561</v>
+        <v>10.1682</v>
       </c>
     </row>
     <row r="126">
@@ -6469,10 +6469,10 @@
         <v>0.82</v>
       </c>
       <c r="I126" t="n">
-        <v>-0.649</v>
+        <v>-0.5936</v>
       </c>
       <c r="J126" t="n">
-        <v>-17.523</v>
+        <v>-16.0272</v>
       </c>
     </row>
     <row r="127">
@@ -6509,10 +6509,10 @@
         <v>1.44</v>
       </c>
       <c r="I127" t="n">
-        <v>0.7026</v>
+        <v>0.648</v>
       </c>
       <c r="J127" t="n">
-        <v>18.9702</v>
+        <v>17.496</v>
       </c>
     </row>
     <row r="128">
@@ -6549,10 +6549,10 @@
         <v>1.16</v>
       </c>
       <c r="I128" t="n">
-        <v>0.3337</v>
+        <v>0.3565</v>
       </c>
       <c r="J128" t="n">
-        <v>9.0099</v>
+        <v>9.625500000000001</v>
       </c>
     </row>
     <row r="129">
@@ -6589,10 +6589,10 @@
         <v>1.06</v>
       </c>
       <c r="I129" t="n">
-        <v>0.1662</v>
+        <v>0.1677</v>
       </c>
       <c r="J129" t="n">
-        <v>4.4874</v>
+        <v>4.5279</v>
       </c>
     </row>
     <row r="130">
@@ -6629,10 +6629,10 @@
         <v>0.67</v>
       </c>
       <c r="I130" t="n">
-        <v>-0.5543</v>
+        <v>-0.3616</v>
       </c>
       <c r="J130" t="n">
-        <v>-14.9661</v>
+        <v>-9.763199999999999</v>
       </c>
     </row>
     <row r="131">
@@ -6669,10 +6669,10 @@
         <v>0.54</v>
       </c>
       <c r="I131" t="n">
-        <v>-0.714</v>
+        <v>-0.481</v>
       </c>
       <c r="J131" t="n">
-        <v>-19.278</v>
+        <v>-12.987</v>
       </c>
     </row>
     <row r="132">
@@ -6709,10 +6709,10 @@
         <v>1.44</v>
       </c>
       <c r="I132" t="n">
-        <v>1.1182</v>
+        <v>0.7988</v>
       </c>
       <c r="J132" t="n">
-        <v>29.0732</v>
+        <v>20.7688</v>
       </c>
     </row>
     <row r="133">
@@ -6749,10 +6749,10 @@
         <v>1.19</v>
       </c>
       <c r="I133" t="n">
-        <v>0.5358000000000001</v>
+        <v>0.4565</v>
       </c>
       <c r="J133" t="n">
-        <v>13.9308</v>
+        <v>11.869</v>
       </c>
     </row>
     <row r="134">
@@ -6789,10 +6789,10 @@
         <v>1.13</v>
       </c>
       <c r="I134" t="n">
-        <v>0.3445</v>
+        <v>0.3684</v>
       </c>
       <c r="J134" t="n">
-        <v>8.957000000000001</v>
+        <v>9.5784</v>
       </c>
     </row>
     <row r="135">
@@ -6829,10 +6829,10 @@
         <v>1.12</v>
       </c>
       <c r="I135" t="n">
-        <v>0.3149</v>
+        <v>0.3526</v>
       </c>
       <c r="J135" t="n">
-        <v>8.1874</v>
+        <v>9.1676</v>
       </c>
     </row>
     <row r="136">
@@ -6869,10 +6869,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I136" t="n">
-        <v>-0.3478</v>
+        <v>-0.2735</v>
       </c>
       <c r="J136" t="n">
-        <v>-9.0428</v>
+        <v>-7.111</v>
       </c>
     </row>
     <row r="137">
@@ -6909,10 +6909,10 @@
         <v>1.04</v>
       </c>
       <c r="I137" t="n">
-        <v>0.1865</v>
+        <v>0.1696</v>
       </c>
       <c r="J137" t="n">
-        <v>4.849</v>
+        <v>4.4096</v>
       </c>
     </row>
     <row r="138">
@@ -6949,10 +6949,10 @@
         <v>0.89</v>
       </c>
       <c r="I138" t="n">
-        <v>-0.1514</v>
+        <v>-0.1269</v>
       </c>
       <c r="J138" t="n">
-        <v>-3.9364</v>
+        <v>-3.2994</v>
       </c>
     </row>
     <row r="139">
@@ -6989,10 +6989,10 @@
         <v>0.89</v>
       </c>
       <c r="I139" t="n">
-        <v>-0.1514</v>
+        <v>-0.1269</v>
       </c>
       <c r="J139" t="n">
-        <v>-3.9364</v>
+        <v>-3.2994</v>
       </c>
     </row>
     <row r="140">
@@ -7029,10 +7029,10 @@
         <v>0.75</v>
       </c>
       <c r="I140" t="n">
-        <v>-0.405</v>
+        <v>-0.2663</v>
       </c>
       <c r="J140" t="n">
-        <v>-10.53</v>
+        <v>-6.9238</v>
       </c>
     </row>
     <row r="141">
@@ -7069,10 +7069,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I141" t="n">
-        <v>-0.6651</v>
+        <v>-0.4455</v>
       </c>
       <c r="J141" t="n">
-        <v>-17.2926</v>
+        <v>-11.583</v>
       </c>
     </row>
     <row r="142">
@@ -7109,10 +7109,10 @@
         <v>1.66</v>
       </c>
       <c r="I142" t="n">
-        <v>1.4335</v>
+        <v>1.0194</v>
       </c>
       <c r="J142" t="n">
-        <v>25.803</v>
+        <v>18.3492</v>
       </c>
     </row>
     <row r="143">
@@ -7149,10 +7149,10 @@
         <v>1.54</v>
       </c>
       <c r="I143" t="n">
-        <v>1.2004</v>
+        <v>0.8768</v>
       </c>
       <c r="J143" t="n">
-        <v>21.6072</v>
+        <v>15.7824</v>
       </c>
     </row>
     <row r="144">
@@ -7189,10 +7189,10 @@
         <v>1.42</v>
       </c>
       <c r="I144" t="n">
-        <v>0.9368</v>
+        <v>0.7325</v>
       </c>
       <c r="J144" t="n">
-        <v>16.8624</v>
+        <v>13.185</v>
       </c>
     </row>
     <row r="145">
@@ -7229,10 +7229,10 @@
         <v>1.31</v>
       </c>
       <c r="I145" t="n">
-        <v>0.6675</v>
+        <v>0.5945</v>
       </c>
       <c r="J145" t="n">
-        <v>12.015</v>
+        <v>10.701</v>
       </c>
     </row>
     <row r="146">
@@ -7269,10 +7269,10 @@
         <v>1.13</v>
       </c>
       <c r="I146" t="n">
-        <v>0.2393</v>
+        <v>0.333</v>
       </c>
       <c r="J146" t="n">
-        <v>4.3074</v>
+        <v>5.994</v>
       </c>
     </row>
     <row r="147">
@@ -7309,10 +7309,10 @@
         <v>0.87</v>
       </c>
       <c r="I147" t="n">
-        <v>-0.0538</v>
+        <v>-0.0732</v>
       </c>
       <c r="J147" t="n">
-        <v>-0.9684</v>
+        <v>-1.3176</v>
       </c>
     </row>
     <row r="148">
@@ -7349,10 +7349,10 @@
         <v>0.7</v>
       </c>
       <c r="I148" t="n">
-        <v>-0.3209</v>
+        <v>-0.2685</v>
       </c>
       <c r="J148" t="n">
-        <v>-5.7762</v>
+        <v>-4.833</v>
       </c>
     </row>
     <row r="149">
@@ -7389,10 +7389,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I149" t="n">
-        <v>-0.5611</v>
+        <v>-0.4038</v>
       </c>
       <c r="J149" t="n">
-        <v>-10.0998</v>
+        <v>-7.2684</v>
       </c>
     </row>
     <row r="150">
@@ -7429,10 +7429,10 @@
         <v>0.35</v>
       </c>
       <c r="I150" t="n">
-        <v>-0.8702</v>
+        <v>-0.6019</v>
       </c>
       <c r="J150" t="n">
-        <v>-15.6636</v>
+        <v>-10.8342</v>
       </c>
     </row>
     <row r="151">
@@ -7469,10 +7469,10 @@
         <v>0.35</v>
       </c>
       <c r="I151" t="n">
-        <v>-0.8702</v>
+        <v>-0.6019</v>
       </c>
       <c r="J151" t="n">
-        <v>-15.6636</v>
+        <v>-10.8342</v>
       </c>
     </row>
     <row r="152">
@@ -7509,10 +7509,10 @@
         <v>1.29</v>
       </c>
       <c r="I152" t="n">
-        <v>0.7658</v>
+        <v>0.5905</v>
       </c>
       <c r="J152" t="n">
-        <v>16.8476</v>
+        <v>12.991</v>
       </c>
     </row>
     <row r="153">
@@ -7549,10 +7549,10 @@
         <v>1.29</v>
       </c>
       <c r="I153" t="n">
-        <v>0.7658</v>
+        <v>0.5905</v>
       </c>
       <c r="J153" t="n">
-        <v>16.8476</v>
+        <v>12.991</v>
       </c>
     </row>
     <row r="154">
@@ -7589,10 +7589,10 @@
         <v>1.18</v>
       </c>
       <c r="I154" t="n">
-        <v>0.4596</v>
+        <v>0.4387</v>
       </c>
       <c r="J154" t="n">
-        <v>10.1112</v>
+        <v>9.651400000000001</v>
       </c>
     </row>
     <row r="155">
@@ -7629,10 +7629,10 @@
         <v>1.17</v>
       </c>
       <c r="I155" t="n">
-        <v>0.4313</v>
+        <v>0.4242</v>
       </c>
       <c r="J155" t="n">
-        <v>9.4886</v>
+        <v>9.3324</v>
       </c>
     </row>
     <row r="156">
@@ -7669,10 +7669,10 @@
         <v>1.09</v>
       </c>
       <c r="I156" t="n">
-        <v>0.2051</v>
+        <v>0.273</v>
       </c>
       <c r="J156" t="n">
-        <v>4.5122</v>
+        <v>6.006</v>
       </c>
     </row>
     <row r="157">
@@ -7709,10 +7709,10 @@
         <v>0.82</v>
       </c>
       <c r="I157" t="n">
-        <v>-0.2123</v>
+        <v>-0.1812</v>
       </c>
       <c r="J157" t="n">
-        <v>-4.6706</v>
+        <v>-3.9864</v>
       </c>
     </row>
     <row r="158">
@@ -7749,10 +7749,10 @@
         <v>0.8</v>
       </c>
       <c r="I158" t="n">
-        <v>-0.2446</v>
+        <v>-0.2022</v>
       </c>
       <c r="J158" t="n">
-        <v>-5.3812</v>
+        <v>-4.4484</v>
       </c>
     </row>
     <row r="159">
@@ -7789,10 +7789,10 @@
         <v>0.75</v>
       </c>
       <c r="I159" t="n">
-        <v>-0.3263</v>
+        <v>-0.2525</v>
       </c>
       <c r="J159" t="n">
-        <v>-7.1786</v>
+        <v>-5.555</v>
       </c>
     </row>
     <row r="160">
@@ -7829,10 +7829,10 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="I160" t="n">
-        <v>-0.4422</v>
+        <v>-0.3073</v>
       </c>
       <c r="J160" t="n">
-        <v>-9.728400000000001</v>
+        <v>-6.7606</v>
       </c>
     </row>
     <row r="161">
@@ -7869,10 +7869,10 @@
         <v>0.49</v>
       </c>
       <c r="I161" t="n">
-        <v>-0.7275</v>
+        <v>-0.4937</v>
       </c>
       <c r="J161" t="n">
-        <v>-16.005</v>
+        <v>-10.8614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: 双向距离 ordered 口径 (α=0.33) 精调定案 — obj 161.86 (+4.24)
ordered 从二值前缀包含改为双向距离加权: 每点 score=max(0,1-0.33|d|),
提前/挤出对称惩罚。新口径下全局 CMA 收敛低于锚点, 局部精调 (seed62/63)
才是爬峰唯一手段。演进: 157.62(旧定案)→精调1 160.82→精调2 161.8643。

权衡: in_topn 85.2%→86.3% (+20人), ordered 66.2%→69.4%, mvp 204→203 (-1),
mismatch 258.9→258.3。2026 关键: 8301 Major mvp 挽回+ord 9/11, 8240 ord 2/7→4/7,
8246 唯一回退 (2/2→1/2)。42 参数写回 EVP_CONFIG, 重建 global_stats/透视表/255赛事明细。

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/event/1608/event_1608_evp_summary.xlsx
+++ b/database/event/1608/event_1608_evp_summary.xlsx
@@ -496,31 +496,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.8247</v>
+        <v>5.7967</v>
       </c>
       <c r="C2" t="n">
-        <v>1.0613</v>
+        <v>1.0562</v>
       </c>
       <c r="D2" t="n">
-        <v>1.9915</v>
+        <v>2.0146</v>
       </c>
       <c r="E2" t="n">
-        <v>5.8247</v>
+        <v>5.7967</v>
       </c>
       <c r="F2" t="n">
-        <v>2.2893</v>
+        <v>2.1924</v>
       </c>
       <c r="G2" t="n">
-        <v>3.5354</v>
+        <v>3.6043</v>
       </c>
       <c r="H2" t="n">
-        <v>2.5797</v>
+        <v>2.3395</v>
       </c>
       <c r="I2" t="n">
-        <v>1.3413</v>
+        <v>1.2633</v>
       </c>
       <c r="J2" t="n">
-        <v>3.5354</v>
+        <v>3.6043</v>
       </c>
       <c r="K2" t="n">
         <v>151</v>
@@ -529,7 +529,7 @@
         <v>131</v>
       </c>
       <c r="M2" t="n">
-        <v>4.8767</v>
+        <v>4.867599999999999</v>
       </c>
       <c r="N2" t="n">
         <v>282</v>
@@ -542,31 +542,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.0961</v>
+        <v>4.128</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7463</v>
+        <v>0.7521</v>
       </c>
       <c r="D3" t="n">
-        <v>1.2112</v>
+        <v>1.2549</v>
       </c>
       <c r="E3" t="n">
-        <v>4.0961</v>
+        <v>4.128</v>
       </c>
       <c r="F3" t="n">
-        <v>2.4452</v>
+        <v>2.3656</v>
       </c>
       <c r="G3" t="n">
-        <v>1.6509</v>
+        <v>1.7624</v>
       </c>
       <c r="H3" t="n">
-        <v>3.1289</v>
+        <v>2.9108</v>
       </c>
       <c r="I3" t="n">
-        <v>1.6269</v>
+        <v>1.5718</v>
       </c>
       <c r="J3" t="n">
-        <v>1.6509</v>
+        <v>1.7624</v>
       </c>
       <c r="K3" t="n">
         <v>80</v>
@@ -575,7 +575,7 @@
         <v>118</v>
       </c>
       <c r="M3" t="n">
-        <v>3.2778</v>
+        <v>3.3342</v>
       </c>
       <c r="N3" t="n">
         <v>198</v>
@@ -588,31 +588,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.9105</v>
+        <v>3.8348</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7125</v>
+        <v>0.6987</v>
       </c>
       <c r="D4" t="n">
-        <v>1.1274</v>
+        <v>1.1215</v>
       </c>
       <c r="E4" t="n">
-        <v>3.9105</v>
+        <v>3.8348</v>
       </c>
       <c r="F4" t="n">
-        <v>4.1605</v>
+        <v>4.0478</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.25</v>
+        <v>-0.213</v>
       </c>
       <c r="H4" t="n">
-        <v>9.172700000000001</v>
+        <v>8.460900000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>4.7694</v>
+        <v>4.5688</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.25</v>
+        <v>-0.213</v>
       </c>
       <c r="K4" t="n">
         <v>151</v>
@@ -621,7 +621,7 @@
         <v>131</v>
       </c>
       <c r="M4" t="n">
-        <v>4.5194</v>
+        <v>4.3558</v>
       </c>
       <c r="N4" t="n">
         <v>282</v>
@@ -630,35 +630,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GeT_RiGhT</t>
+          <t>f0rest</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.5759</v>
+        <v>3.5577</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6515</v>
+        <v>0.6482</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9762999999999999</v>
+        <v>0.9953</v>
       </c>
       <c r="E5" t="n">
-        <v>3.5759</v>
+        <v>3.5577</v>
       </c>
       <c r="F5" t="n">
-        <v>1.7565</v>
+        <v>2.6078</v>
       </c>
       <c r="G5" t="n">
-        <v>1.8194</v>
+        <v>0.9499</v>
       </c>
       <c r="H5" t="n">
-        <v>1.7565</v>
+        <v>3.7099</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9133</v>
+        <v>2.0033</v>
       </c>
       <c r="J5" t="n">
-        <v>1.8194</v>
+        <v>0.9499</v>
       </c>
       <c r="K5" t="n">
         <v>80</v>
@@ -667,7 +667,7 @@
         <v>118</v>
       </c>
       <c r="M5" t="n">
-        <v>2.7327</v>
+        <v>2.9532</v>
       </c>
       <c r="N5" t="n">
         <v>198</v>
@@ -676,35 +676,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>f0rest</t>
+          <t>GeT_RiGhT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.5648</v>
+        <v>3.547</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6495</v>
+        <v>0.6463</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9905</v>
       </c>
       <c r="E6" t="n">
-        <v>3.5648</v>
+        <v>3.547</v>
       </c>
       <c r="F6" t="n">
-        <v>2.7084</v>
+        <v>1.6213</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8564000000000001</v>
+        <v>1.9257</v>
       </c>
       <c r="H6" t="n">
-        <v>4.0563</v>
+        <v>1.6213</v>
       </c>
       <c r="I6" t="n">
-        <v>2.1091</v>
+        <v>0.8754999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8564000000000001</v>
+        <v>1.9257</v>
       </c>
       <c r="K6" t="n">
         <v>80</v>
@@ -713,7 +713,7 @@
         <v>118</v>
       </c>
       <c r="M6" t="n">
-        <v>2.9655</v>
+        <v>2.8012</v>
       </c>
       <c r="N6" t="n">
         <v>198</v>
@@ -726,31 +726,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.2144</v>
+        <v>2.0905</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4035</v>
+        <v>0.3809</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3617</v>
+        <v>0.3274</v>
       </c>
       <c r="E7" t="n">
-        <v>2.2144</v>
+        <v>2.0905</v>
       </c>
       <c r="F7" t="n">
-        <v>2.7994</v>
+        <v>2.7174</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.585</v>
+        <v>-0.6269</v>
       </c>
       <c r="H7" t="n">
-        <v>4.3769</v>
+        <v>4.0715</v>
       </c>
       <c r="I7" t="n">
-        <v>2.2758</v>
+        <v>2.1986</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.585</v>
+        <v>-0.6269</v>
       </c>
       <c r="K7" t="n">
         <v>143</v>
@@ -759,7 +759,7 @@
         <v>40</v>
       </c>
       <c r="M7" t="n">
-        <v>1.6908</v>
+        <v>1.5717</v>
       </c>
       <c r="N7" t="n">
         <v>183</v>
@@ -772,31 +772,31 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.2571</v>
+        <v>1.0133</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2291</v>
+        <v>0.1846</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.07049999999999999</v>
+        <v>-0.1629</v>
       </c>
       <c r="E8" t="n">
-        <v>1.2571</v>
+        <v>1.0133</v>
       </c>
       <c r="F8" t="n">
-        <v>2.1115</v>
+        <v>1.8943</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.8544</v>
+        <v>-0.881</v>
       </c>
       <c r="H8" t="n">
-        <v>2.1115</v>
+        <v>1.8943</v>
       </c>
       <c r="I8" t="n">
-        <v>1.0979</v>
+        <v>1.0229</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.8544</v>
+        <v>-0.881</v>
       </c>
       <c r="K8" t="n">
         <v>143</v>
@@ -805,7 +805,7 @@
         <v>40</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2435</v>
+        <v>0.1418999999999999</v>
       </c>
       <c r="N8" t="n">
         <v>183</v>
@@ -818,31 +818,31 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6732</v>
+        <v>0.5793</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1227</v>
+        <v>0.1056</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.3341</v>
+        <v>-0.3605</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6732</v>
+        <v>0.5793</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7718</v>
+        <v>0.6887</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.1094</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7718</v>
+        <v>0.6887</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4013</v>
+        <v>0.3719</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.1094</v>
       </c>
       <c r="K9" t="n">
         <v>72</v>
@@ -851,7 +851,7 @@
         <v>53</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3027</v>
+        <v>0.2625</v>
       </c>
       <c r="N9" t="n">
         <v>125</v>
@@ -864,31 +864,31 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.4997</v>
+        <v>0.5508999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>0.091</v>
+        <v>0.1004</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.4124</v>
+        <v>-0.3734</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4997</v>
+        <v>0.5508999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5193</v>
+        <v>0.4472</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0196</v>
+        <v>0.1037</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5193</v>
+        <v>0.4472</v>
       </c>
       <c r="I10" t="n">
-        <v>0.27</v>
+        <v>0.2415</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.0196</v>
+        <v>0.1037</v>
       </c>
       <c r="K10" t="n">
         <v>151</v>
@@ -897,7 +897,7 @@
         <v>131</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2504</v>
+        <v>0.3452</v>
       </c>
       <c r="N10" t="n">
         <v>282</v>
@@ -906,35 +906,35 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JW</t>
+          <t>dennis</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.4333</v>
+        <v>0.5093</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0789</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.4424</v>
+        <v>-0.3924</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4333</v>
+        <v>0.5093</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.6487000000000001</v>
+        <v>-0.6006</v>
       </c>
       <c r="G11" t="n">
-        <v>1.082</v>
+        <v>1.1099</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.6487000000000001</v>
+        <v>-0.6006</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.3373</v>
+        <v>-0.3243</v>
       </c>
       <c r="J11" t="n">
-        <v>1.082</v>
+        <v>1.1099</v>
       </c>
       <c r="K11" t="n">
         <v>151</v>
@@ -943,7 +943,7 @@
         <v>131</v>
       </c>
       <c r="M11" t="n">
-        <v>0.7447000000000001</v>
+        <v>0.7856000000000001</v>
       </c>
       <c r="N11" t="n">
         <v>282</v>
@@ -952,35 +952,35 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dennis</t>
+          <t>JW</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.4126</v>
+        <v>0.3452</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0752</v>
+        <v>0.0629</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.4517</v>
+        <v>-0.4671</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4126</v>
+        <v>0.3452</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.6197</v>
+        <v>-0.7246</v>
       </c>
       <c r="G12" t="n">
-        <v>1.0323</v>
+        <v>1.0698</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.6197</v>
+        <v>-0.7246</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.3222</v>
+        <v>-0.3913</v>
       </c>
       <c r="J12" t="n">
-        <v>1.0323</v>
+        <v>1.0698</v>
       </c>
       <c r="K12" t="n">
         <v>151</v>
@@ -989,7 +989,7 @@
         <v>131</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7101</v>
+        <v>0.6785000000000001</v>
       </c>
       <c r="N12" t="n">
         <v>282</v>
@@ -998,93 +998,93 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dupreeh</t>
+          <t>Xizt</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.2348</v>
+        <v>0.2641</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0428</v>
+        <v>0.0481</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.532</v>
+        <v>-0.504</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2348</v>
+        <v>0.2641</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0323</v>
+        <v>-1.0845</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2025</v>
+        <v>1.3486</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0323</v>
+        <v>-1.0845</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0168</v>
+        <v>-0.5856</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2025</v>
+        <v>1.3486</v>
       </c>
       <c r="K13" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L13" t="n">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2193</v>
+        <v>0.763</v>
       </c>
       <c r="N13" t="n">
-        <v>125</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Xizt</t>
+          <t>dupreeh</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0154</v>
+        <v>0.2324</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0028</v>
+        <v>0.0423</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.6311</v>
+        <v>-0.5184</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0154</v>
+        <v>0.2324</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.1905</v>
+        <v>-0.0322</v>
       </c>
       <c r="G14" t="n">
-        <v>1.2059</v>
+        <v>0.2646</v>
       </c>
       <c r="H14" t="n">
-        <v>-1.1905</v>
+        <v>-0.0322</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.619</v>
+        <v>-0.0174</v>
       </c>
       <c r="J14" t="n">
-        <v>1.2059</v>
+        <v>0.2646</v>
       </c>
       <c r="K14" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="L14" t="n">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="M14" t="n">
-        <v>0.5869</v>
+        <v>0.2472</v>
       </c>
       <c r="N14" t="n">
-        <v>198</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15">
@@ -1094,31 +1094,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.3853</v>
+        <v>-0.3294</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.0702</v>
+        <v>-0.06</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.8120000000000001</v>
+        <v>-0.7742</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.3853</v>
+        <v>-0.3294</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.6149</v>
+        <v>-0.5552</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2296</v>
+        <v>0.2258</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.6149</v>
+        <v>-0.5552</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.3197</v>
+        <v>-0.2998</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2296</v>
+        <v>0.2258</v>
       </c>
       <c r="K15" t="n">
         <v>72</v>
@@ -1127,7 +1127,7 @@
         <v>53</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.09009999999999999</v>
+        <v>-0.07400000000000001</v>
       </c>
       <c r="N15" t="n">
         <v>125</v>
@@ -1140,31 +1140,31 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.3872</v>
+        <v>-0.5877</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.0706</v>
+        <v>-0.1071</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.8128</v>
+        <v>-0.8917</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.3872</v>
+        <v>-0.5877</v>
       </c>
       <c r="F16" t="n">
-        <v>0.522</v>
+        <v>0.347</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.9092</v>
+        <v>-0.9347</v>
       </c>
       <c r="H16" t="n">
-        <v>0.522</v>
+        <v>0.347</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2714</v>
+        <v>0.1874</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.9092</v>
+        <v>-0.9347</v>
       </c>
       <c r="K16" t="n">
         <v>143</v>
@@ -1173,7 +1173,7 @@
         <v>40</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.6378</v>
+        <v>-0.7473</v>
       </c>
       <c r="N16" t="n">
         <v>183</v>
@@ -1186,31 +1186,31 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.7385</v>
+        <v>-0.9546</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.1346</v>
+        <v>-0.1739</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.9714</v>
+        <v>-1.0588</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.7385</v>
+        <v>-0.9546</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.4631</v>
+        <v>-0.6235000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.2754</v>
+        <v>-0.3311</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.4631</v>
+        <v>-0.6235000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.2408</v>
+        <v>-0.3367</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.2754</v>
+        <v>-0.3311</v>
       </c>
       <c r="K17" t="n">
         <v>143</v>
@@ -1219,7 +1219,7 @@
         <v>40</v>
       </c>
       <c r="M17" t="n">
-        <v>-0.5162</v>
+        <v>-0.6677999999999999</v>
       </c>
       <c r="N17" t="n">
         <v>183</v>
@@ -1232,31 +1232,31 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-1.319</v>
+        <v>-1.3182</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.2403</v>
+        <v>-0.2402</v>
       </c>
       <c r="D18" t="n">
-        <v>-1.2335</v>
+        <v>-1.2243</v>
       </c>
       <c r="E18" t="n">
-        <v>-1.319</v>
+        <v>-1.3182</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.0076</v>
+        <v>-0.9948</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.3114</v>
+        <v>-0.3234</v>
       </c>
       <c r="H18" t="n">
-        <v>-1.0076</v>
+        <v>-0.9948</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.5239</v>
+        <v>-0.5372</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.3114</v>
+        <v>-0.3234</v>
       </c>
       <c r="K18" t="n">
         <v>72</v>
@@ -1265,7 +1265,7 @@
         <v>53</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.8353</v>
+        <v>-0.8606</v>
       </c>
       <c r="N18" t="n">
         <v>125</v>
@@ -1278,31 +1278,31 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-1.5251</v>
+        <v>-1.5186</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.2779</v>
+        <v>-0.2767</v>
       </c>
       <c r="D19" t="n">
-        <v>-1.3265</v>
+        <v>-1.3155</v>
       </c>
       <c r="E19" t="n">
-        <v>-1.5251</v>
+        <v>-1.5186</v>
       </c>
       <c r="F19" t="n">
-        <v>-1.0366</v>
+        <v>-1.0017</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.4885</v>
+        <v>-0.5169</v>
       </c>
       <c r="H19" t="n">
-        <v>-1.0366</v>
+        <v>-1.0017</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.539</v>
+        <v>-0.5409</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.4885</v>
+        <v>-0.5169</v>
       </c>
       <c r="K19" t="n">
         <v>72</v>
@@ -1311,7 +1311,7 @@
         <v>53</v>
       </c>
       <c r="M19" t="n">
-        <v>-1.0275</v>
+        <v>-1.0578</v>
       </c>
       <c r="N19" t="n">
         <v>125</v>
@@ -1324,31 +1324,31 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-1.8139</v>
+        <v>-1.5637</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.3305</v>
+        <v>-0.2849</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.4569</v>
+        <v>-1.336</v>
       </c>
       <c r="E20" t="n">
-        <v>-1.8139</v>
+        <v>-1.5637</v>
       </c>
       <c r="F20" t="n">
-        <v>-2.2708</v>
+        <v>-2.0721</v>
       </c>
       <c r="G20" t="n">
-        <v>0.4569</v>
+        <v>0.5084</v>
       </c>
       <c r="H20" t="n">
-        <v>-2.2708</v>
+        <v>-2.0721</v>
       </c>
       <c r="I20" t="n">
-        <v>-1.1807</v>
+        <v>-1.1189</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4569</v>
+        <v>0.5084</v>
       </c>
       <c r="K20" t="n">
         <v>80</v>
@@ -1357,7 +1357,7 @@
         <v>118</v>
       </c>
       <c r="M20" t="n">
-        <v>-0.7238000000000001</v>
+        <v>-0.6105</v>
       </c>
       <c r="N20" t="n">
         <v>198</v>
@@ -1370,31 +1370,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-2.9582</v>
+        <v>-2.9121</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.539</v>
+        <v>-0.5306</v>
       </c>
       <c r="D21" t="n">
-        <v>-1.9735</v>
+        <v>-1.9499</v>
       </c>
       <c r="E21" t="n">
-        <v>-2.9582</v>
+        <v>-2.9121</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.196</v>
+        <v>-2.113</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.7622</v>
+        <v>-0.7991</v>
       </c>
       <c r="H21" t="n">
-        <v>-2.196</v>
+        <v>-2.113</v>
       </c>
       <c r="I21" t="n">
-        <v>-1.1418</v>
+        <v>-1.141</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.7622</v>
+        <v>-0.7991</v>
       </c>
       <c r="K21" t="n">
         <v>143</v>
@@ -1403,7 +1403,7 @@
         <v>40</v>
       </c>
       <c r="M21" t="n">
-        <v>-1.904</v>
+        <v>-1.9401</v>
       </c>
       <c r="N21" t="n">
         <v>183</v>
@@ -1509,10 +1509,10 @@
         <v>1.14</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4503</v>
+        <v>0.4199</v>
       </c>
       <c r="J2" t="n">
-        <v>11.2575</v>
+        <v>10.4975</v>
       </c>
     </row>
     <row r="3">
@@ -1549,10 +1549,10 @@
         <v>0.74</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.265</v>
+        <v>-0.2849</v>
       </c>
       <c r="J3" t="n">
-        <v>-6.625</v>
+        <v>-7.1225</v>
       </c>
     </row>
     <row r="4">
@@ -1589,10 +1589,10 @@
         <v>0.67</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.3292</v>
+        <v>-0.3474</v>
       </c>
       <c r="J4" t="n">
-        <v>-8.23</v>
+        <v>-8.685</v>
       </c>
     </row>
     <row r="5">
@@ -1629,10 +1629,10 @@
         <v>0.6</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.3947</v>
+        <v>-0.4101</v>
       </c>
       <c r="J5" t="n">
-        <v>-9.8675</v>
+        <v>-10.2525</v>
       </c>
     </row>
     <row r="6">
@@ -1669,10 +1669,10 @@
         <v>0.52</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.4694</v>
+        <v>-0.4807</v>
       </c>
       <c r="J6" t="n">
-        <v>-11.735</v>
+        <v>-12.0175</v>
       </c>
     </row>
     <row r="7">
@@ -1709,10 +1709,10 @@
         <v>1.54</v>
       </c>
       <c r="I7" t="n">
-        <v>1.1806</v>
+        <v>1.1994</v>
       </c>
       <c r="J7" t="n">
-        <v>29.515</v>
+        <v>29.985</v>
       </c>
     </row>
     <row r="8">
@@ -1749,10 +1749,10 @@
         <v>1.32</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8266</v>
+        <v>0.7844</v>
       </c>
       <c r="J8" t="n">
-        <v>20.665</v>
+        <v>19.61</v>
       </c>
     </row>
     <row r="9">
@@ -1789,10 +1789,10 @@
         <v>1.23</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6236</v>
+        <v>0.6039</v>
       </c>
       <c r="J9" t="n">
-        <v>15.59</v>
+        <v>15.0975</v>
       </c>
     </row>
     <row r="10">
@@ -1829,10 +1829,10 @@
         <v>1.08</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2333</v>
+        <v>0.2487</v>
       </c>
       <c r="J10" t="n">
-        <v>5.8325</v>
+        <v>6.2175</v>
       </c>
     </row>
     <row r="11">
@@ -1869,10 +1869,10 @@
         <v>1.07</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2033</v>
+        <v>0.2206</v>
       </c>
       <c r="J11" t="n">
-        <v>5.0825</v>
+        <v>5.515</v>
       </c>
     </row>
     <row r="12">
@@ -1909,10 +1909,10 @@
         <v>1.44</v>
       </c>
       <c r="I12" t="n">
-        <v>0.5652</v>
+        <v>0.5692</v>
       </c>
       <c r="J12" t="n">
-        <v>14.13</v>
+        <v>14.23</v>
       </c>
     </row>
     <row r="13">
@@ -1949,10 +1949,10 @@
         <v>1.29</v>
       </c>
       <c r="I13" t="n">
-        <v>0.393</v>
+        <v>0.4061</v>
       </c>
       <c r="J13" t="n">
-        <v>9.824999999999999</v>
+        <v>10.1525</v>
       </c>
     </row>
     <row r="14">
@@ -1989,10 +1989,10 @@
         <v>1.24</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3335</v>
+        <v>0.3488</v>
       </c>
       <c r="J14" t="n">
-        <v>8.3375</v>
+        <v>8.720000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -2029,10 +2029,10 @@
         <v>1.06</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0973</v>
+        <v>0.1131</v>
       </c>
       <c r="J15" t="n">
-        <v>2.4325</v>
+        <v>2.8275</v>
       </c>
     </row>
     <row r="16">
@@ -2069,10 +2069,10 @@
         <v>0.78</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.276</v>
+        <v>-0.2855</v>
       </c>
       <c r="J16" t="n">
-        <v>-6.9</v>
+        <v>-7.1375</v>
       </c>
     </row>
     <row r="17">
@@ -2109,10 +2109,10 @@
         <v>1.34</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6261</v>
+        <v>0.5936</v>
       </c>
       <c r="J17" t="n">
-        <v>15.6525</v>
+        <v>14.84</v>
       </c>
     </row>
     <row r="18">
@@ -2149,10 +2149,10 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0527</v>
+        <v>0.0392</v>
       </c>
       <c r="J18" t="n">
-        <v>1.3175</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="19">
@@ -2189,10 +2189,10 @@
         <v>0.62</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.3822</v>
+        <v>-0.3971</v>
       </c>
       <c r="J19" t="n">
-        <v>-9.555</v>
+        <v>-9.9275</v>
       </c>
     </row>
     <row r="20">
@@ -2229,10 +2229,10 @@
         <v>0.59</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.4102</v>
+        <v>-0.4238</v>
       </c>
       <c r="J20" t="n">
-        <v>-10.255</v>
+        <v>-10.595</v>
       </c>
     </row>
     <row r="21">
@@ -2269,10 +2269,10 @@
         <v>0.32</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.6588000000000001</v>
+        <v>-0.6564</v>
       </c>
       <c r="J21" t="n">
-        <v>-16.47</v>
+        <v>-16.41</v>
       </c>
     </row>
     <row r="22">
@@ -2309,10 +2309,10 @@
         <v>1.26</v>
       </c>
       <c r="I22" t="n">
-        <v>0.5706</v>
+        <v>0.5508</v>
       </c>
       <c r="J22" t="n">
-        <v>15.9768</v>
+        <v>15.4224</v>
       </c>
     </row>
     <row r="23">
@@ -2349,10 +2349,10 @@
         <v>1.03</v>
       </c>
       <c r="I23" t="n">
-        <v>0.105</v>
+        <v>0.1095</v>
       </c>
       <c r="J23" t="n">
-        <v>2.94</v>
+        <v>3.066</v>
       </c>
     </row>
     <row r="24">
@@ -2389,10 +2389,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.0829</v>
+        <v>-0.095</v>
       </c>
       <c r="J24" t="n">
-        <v>-2.3212</v>
+        <v>-2.66</v>
       </c>
     </row>
     <row r="25">
@@ -2429,10 +2429,10 @@
         <v>0.88</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.1494</v>
+        <v>-0.1641</v>
       </c>
       <c r="J25" t="n">
-        <v>-4.1832</v>
+        <v>-4.5948</v>
       </c>
     </row>
     <row r="26">
@@ -2469,10 +2469,10 @@
         <v>0.59</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.4319</v>
+        <v>-0.4408</v>
       </c>
       <c r="J26" t="n">
-        <v>-12.0932</v>
+        <v>-12.3424</v>
       </c>
     </row>
     <row r="27">
@@ -2509,10 +2509,10 @@
         <v>1.44</v>
       </c>
       <c r="I27" t="n">
-        <v>1.1096</v>
+        <v>1.0814</v>
       </c>
       <c r="J27" t="n">
-        <v>31.0688</v>
+        <v>30.2792</v>
       </c>
     </row>
     <row r="28">
@@ -2549,10 +2549,10 @@
         <v>1.18</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5533</v>
+        <v>0.53</v>
       </c>
       <c r="J28" t="n">
-        <v>15.4924</v>
+        <v>14.84</v>
       </c>
     </row>
     <row r="29">
@@ -2589,10 +2589,10 @@
         <v>0.98</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.1025</v>
+        <v>-0.1056</v>
       </c>
       <c r="J29" t="n">
-        <v>-2.87</v>
+        <v>-2.9568</v>
       </c>
     </row>
     <row r="30">
@@ -2629,10 +2629,10 @@
         <v>0.96</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.1742</v>
+        <v>-0.1755</v>
       </c>
       <c r="J30" t="n">
-        <v>-4.8776</v>
+        <v>-4.914</v>
       </c>
     </row>
     <row r="31">
@@ -2669,10 +2669,10 @@
         <v>0.63</v>
       </c>
       <c r="I31" t="n">
-        <v>-1.054</v>
+        <v>-0.9631999999999999</v>
       </c>
       <c r="J31" t="n">
-        <v>-29.512</v>
+        <v>-26.9696</v>
       </c>
     </row>
     <row r="32">
@@ -2709,10 +2709,10 @@
         <v>1.78</v>
       </c>
       <c r="I32" t="n">
-        <v>0.9325</v>
+        <v>0.9091</v>
       </c>
       <c r="J32" t="n">
-        <v>26.11</v>
+        <v>25.4548</v>
       </c>
     </row>
     <row r="33">
@@ -2749,10 +2749,10 @@
         <v>1.19</v>
       </c>
       <c r="I33" t="n">
-        <v>0.2729</v>
+        <v>0.2896</v>
       </c>
       <c r="J33" t="n">
-        <v>7.6412</v>
+        <v>8.1088</v>
       </c>
     </row>
     <row r="34">
@@ -2789,10 +2789,10 @@
         <v>1.04</v>
       </c>
       <c r="I34" t="n">
-        <v>0.065</v>
+        <v>0.0794</v>
       </c>
       <c r="J34" t="n">
-        <v>1.82</v>
+        <v>2.2232</v>
       </c>
     </row>
     <row r="35">
@@ -2829,10 +2829,10 @@
         <v>1.03</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0475</v>
+        <v>0.061</v>
       </c>
       <c r="J35" t="n">
-        <v>1.33</v>
+        <v>1.708</v>
       </c>
     </row>
     <row r="36">
@@ -2869,10 +2869,10 @@
         <v>0.76</v>
       </c>
       <c r="I36" t="n">
-        <v>-0.2953</v>
+        <v>-0.3045</v>
       </c>
       <c r="J36" t="n">
-        <v>-8.2684</v>
+        <v>-8.526</v>
       </c>
     </row>
     <row r="37">
@@ -2909,10 +2909,10 @@
         <v>1.44</v>
       </c>
       <c r="I37" t="n">
-        <v>0.6849</v>
+        <v>0.6587</v>
       </c>
       <c r="J37" t="n">
-        <v>19.1772</v>
+        <v>18.4436</v>
       </c>
     </row>
     <row r="38">
@@ -2949,10 +2949,10 @@
         <v>1.14</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2686</v>
+        <v>0.2714</v>
       </c>
       <c r="J38" t="n">
-        <v>7.5208</v>
+        <v>7.5992</v>
       </c>
     </row>
     <row r="39">
@@ -2989,10 +2989,10 @@
         <v>0.86</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.1685</v>
+        <v>-0.1839</v>
       </c>
       <c r="J39" t="n">
-        <v>-4.718</v>
+        <v>-5.1492</v>
       </c>
     </row>
     <row r="40">
@@ -3029,10 +3029,10 @@
         <v>0.85</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.1788</v>
+        <v>-0.1944</v>
       </c>
       <c r="J40" t="n">
-        <v>-5.0064</v>
+        <v>-5.4432</v>
       </c>
     </row>
     <row r="41">
@@ -3069,10 +3069,10 @@
         <v>0.32</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.6715</v>
+        <v>-0.6664</v>
       </c>
       <c r="J41" t="n">
-        <v>-18.802</v>
+        <v>-18.6592</v>
       </c>
     </row>
     <row r="42">
@@ -3109,10 +3109,10 @@
         <v>1.06</v>
       </c>
       <c r="I42" t="n">
-        <v>0.2499</v>
+        <v>0.2347</v>
       </c>
       <c r="J42" t="n">
-        <v>5.2479</v>
+        <v>4.9287</v>
       </c>
     </row>
     <row r="43">
@@ -3149,10 +3149,10 @@
         <v>0.91</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.0922</v>
+        <v>-0.1116</v>
       </c>
       <c r="J43" t="n">
-        <v>-1.9362</v>
+        <v>-2.3436</v>
       </c>
     </row>
     <row r="44">
@@ -3189,10 +3189,10 @@
         <v>0.78</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.2311</v>
+        <v>-0.2506</v>
       </c>
       <c r="J44" t="n">
-        <v>-4.8531</v>
+        <v>-5.2626</v>
       </c>
     </row>
     <row r="45">
@@ -3229,10 +3229,10 @@
         <v>0.62</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.3806</v>
+        <v>-0.3959</v>
       </c>
       <c r="J45" t="n">
-        <v>-7.9926</v>
+        <v>-8.3139</v>
       </c>
     </row>
     <row r="46">
@@ -3269,10 +3269,10 @@
         <v>0.45</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.5387</v>
+        <v>-0.5449000000000001</v>
       </c>
       <c r="J46" t="n">
-        <v>-11.3127</v>
+        <v>-11.4429</v>
       </c>
     </row>
     <row r="47">
@@ -3309,10 +3309,10 @@
         <v>1.47</v>
       </c>
       <c r="I47" t="n">
-        <v>1.1072</v>
+        <v>1.0663</v>
       </c>
       <c r="J47" t="n">
-        <v>23.2512</v>
+        <v>22.3923</v>
       </c>
     </row>
     <row r="48">
@@ -3349,10 +3349,10 @@
         <v>1.4</v>
       </c>
       <c r="I48" t="n">
-        <v>1.0101</v>
+        <v>0.9530999999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>21.2121</v>
+        <v>20.0151</v>
       </c>
     </row>
     <row r="49">
@@ -3389,10 +3389,10 @@
         <v>1.19</v>
       </c>
       <c r="I49" t="n">
-        <v>0.5387</v>
+        <v>0.5253</v>
       </c>
       <c r="J49" t="n">
-        <v>11.3127</v>
+        <v>11.0313</v>
       </c>
     </row>
     <row r="50">
@@ -3429,10 +3429,10 @@
         <v>0.95</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.2459</v>
+        <v>-0.2341</v>
       </c>
       <c r="J50" t="n">
-        <v>-5.1639</v>
+        <v>-4.9161</v>
       </c>
     </row>
     <row r="51">
@@ -3469,10 +3469,10 @@
         <v>0.9</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.3989</v>
+        <v>-0.3769</v>
       </c>
       <c r="J51" t="n">
-        <v>-8.376899999999999</v>
+        <v>-7.9149</v>
       </c>
     </row>
     <row r="52">
@@ -3509,10 +3509,10 @@
         <v>0.85</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.1055</v>
+        <v>-0.1372</v>
       </c>
       <c r="J52" t="n">
-        <v>-2.321</v>
+        <v>-3.0184</v>
       </c>
     </row>
     <row r="53">
@@ -3549,10 +3549,10 @@
         <v>0.78</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.1872</v>
+        <v>-0.2163</v>
       </c>
       <c r="J53" t="n">
-        <v>-4.1184</v>
+        <v>-4.7586</v>
       </c>
     </row>
     <row r="54">
@@ -3589,10 +3589,10 @@
         <v>0.47</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.4897</v>
+        <v>-0.5037</v>
       </c>
       <c r="J54" t="n">
-        <v>-10.7734</v>
+        <v>-11.0814</v>
       </c>
     </row>
     <row r="55">
@@ -3629,10 +3629,10 @@
         <v>0.47</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.4897</v>
+        <v>-0.5037</v>
       </c>
       <c r="J55" t="n">
-        <v>-10.7734</v>
+        <v>-11.0814</v>
       </c>
     </row>
     <row r="56">
@@ -3669,10 +3669,10 @@
         <v>0.34</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.6145</v>
+        <v>-0.6188</v>
       </c>
       <c r="J56" t="n">
-        <v>-13.519</v>
+        <v>-13.6136</v>
       </c>
     </row>
     <row r="57">
@@ -3709,10 +3709,10 @@
         <v>1.84</v>
       </c>
       <c r="I57" t="n">
-        <v>1.4997</v>
+        <v>1.4941</v>
       </c>
       <c r="J57" t="n">
-        <v>32.9934</v>
+        <v>32.8702</v>
       </c>
     </row>
     <row r="58">
@@ -3749,10 +3749,10 @@
         <v>1.64</v>
       </c>
       <c r="I58" t="n">
-        <v>1.2675</v>
+        <v>1.2479</v>
       </c>
       <c r="J58" t="n">
-        <v>27.885</v>
+        <v>27.4538</v>
       </c>
     </row>
     <row r="59">
@@ -3789,10 +3789,10 @@
         <v>1.31</v>
       </c>
       <c r="I59" t="n">
-        <v>0.7738</v>
+        <v>0.7439</v>
       </c>
       <c r="J59" t="n">
-        <v>17.0236</v>
+        <v>16.3658</v>
       </c>
     </row>
     <row r="60">
@@ -3829,10 +3829,10 @@
         <v>1.26</v>
       </c>
       <c r="I60" t="n">
-        <v>0.6592</v>
+        <v>0.6425999999999999</v>
       </c>
       <c r="J60" t="n">
-        <v>14.5024</v>
+        <v>14.1372</v>
       </c>
     </row>
     <row r="61">
@@ -3869,10 +3869,10 @@
         <v>1.07</v>
       </c>
       <c r="I61" t="n">
-        <v>0.1635</v>
+        <v>0.1928</v>
       </c>
       <c r="J61" t="n">
-        <v>3.597</v>
+        <v>4.2416</v>
       </c>
     </row>
     <row r="62">
@@ -3909,10 +3909,10 @@
         <v>1.4</v>
       </c>
       <c r="I62" t="n">
-        <v>1.0249</v>
+        <v>0.9668</v>
       </c>
       <c r="J62" t="n">
-        <v>22.5478</v>
+        <v>21.2696</v>
       </c>
     </row>
     <row r="63">
@@ -3949,10 +3949,10 @@
         <v>1.36</v>
       </c>
       <c r="I63" t="n">
-        <v>0.9524</v>
+        <v>0.8902</v>
       </c>
       <c r="J63" t="n">
-        <v>20.9528</v>
+        <v>19.5844</v>
       </c>
     </row>
     <row r="64">
@@ -3989,10 +3989,10 @@
         <v>1.11</v>
       </c>
       <c r="I64" t="n">
-        <v>0.3455</v>
+        <v>0.3463</v>
       </c>
       <c r="J64" t="n">
-        <v>7.601</v>
+        <v>7.6186</v>
       </c>
     </row>
     <row r="65">
@@ -4029,10 +4029,10 @@
         <v>0.97</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.1639</v>
+        <v>-0.1589</v>
       </c>
       <c r="J65" t="n">
-        <v>-3.6058</v>
+        <v>-3.4958</v>
       </c>
     </row>
     <row r="66">
@@ -4069,10 +4069,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.6317</v>
+        <v>-0.59</v>
       </c>
       <c r="J66" t="n">
-        <v>-13.8974</v>
+        <v>-12.98</v>
       </c>
     </row>
     <row r="67">
@@ -4109,10 +4109,10 @@
         <v>1.29</v>
       </c>
       <c r="I67" t="n">
-        <v>0.7171999999999999</v>
+        <v>0.6686</v>
       </c>
       <c r="J67" t="n">
-        <v>15.7784</v>
+        <v>14.7092</v>
       </c>
     </row>
     <row r="68">
@@ -4149,10 +4149,10 @@
         <v>0.77</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.2418</v>
+        <v>-0.2609</v>
       </c>
       <c r="J68" t="n">
-        <v>-5.3196</v>
+        <v>-5.7398</v>
       </c>
     </row>
     <row r="69">
@@ -4189,10 +4189,10 @@
         <v>0.75</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.2606</v>
+        <v>-0.2794</v>
       </c>
       <c r="J69" t="n">
-        <v>-5.7332</v>
+        <v>-6.1468</v>
       </c>
     </row>
     <row r="70">
@@ -4229,10 +4229,10 @@
         <v>0.73</v>
       </c>
       <c r="I70" t="n">
-        <v>-0.2795</v>
+        <v>-0.2979</v>
       </c>
       <c r="J70" t="n">
-        <v>-6.149</v>
+        <v>-6.5538</v>
       </c>
     </row>
     <row r="71">
@@ -4269,10 +4269,10 @@
         <v>0.37</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.6142</v>
+        <v>-0.6149</v>
       </c>
       <c r="J71" t="n">
-        <v>-13.5124</v>
+        <v>-13.5278</v>
       </c>
     </row>
     <row r="72">
@@ -4309,10 +4309,10 @@
         <v>1.13</v>
       </c>
       <c r="I72" t="n">
-        <v>0.2429</v>
+        <v>0.2489</v>
       </c>
       <c r="J72" t="n">
-        <v>7.287</v>
+        <v>7.467</v>
       </c>
     </row>
     <row r="73">
@@ -4349,10 +4349,10 @@
         <v>1.09</v>
       </c>
       <c r="I73" t="n">
-        <v>0.1804</v>
+        <v>0.1879</v>
       </c>
       <c r="J73" t="n">
-        <v>5.412</v>
+        <v>5.637</v>
       </c>
     </row>
     <row r="74">
@@ -4389,10 +4389,10 @@
         <v>0.97</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.0473</v>
+        <v>-0.0562</v>
       </c>
       <c r="J74" t="n">
-        <v>-1.419</v>
+        <v>-1.686</v>
       </c>
     </row>
     <row r="75">
@@ -4429,10 +4429,10 @@
         <v>0.89</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.141</v>
+        <v>-0.1549</v>
       </c>
       <c r="J75" t="n">
-        <v>-4.23</v>
+        <v>-4.647</v>
       </c>
     </row>
     <row r="76">
@@ -4469,10 +4469,10 @@
         <v>0.73</v>
       </c>
       <c r="I76" t="n">
-        <v>-0.3032</v>
+        <v>-0.3163</v>
       </c>
       <c r="J76" t="n">
-        <v>-9.096</v>
+        <v>-9.489000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -4509,10 +4509,10 @@
         <v>1.74</v>
       </c>
       <c r="I77" t="n">
-        <v>0.9217</v>
+        <v>0.8946</v>
       </c>
       <c r="J77" t="n">
-        <v>27.651</v>
+        <v>26.838</v>
       </c>
     </row>
     <row r="78">
@@ -4549,10 +4549,10 @@
         <v>1.07</v>
       </c>
       <c r="I78" t="n">
-        <v>0.1224</v>
+        <v>0.1362</v>
       </c>
       <c r="J78" t="n">
-        <v>3.672</v>
+        <v>4.086</v>
       </c>
     </row>
     <row r="79">
@@ -4589,10 +4589,10 @@
         <v>0.92</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.1192</v>
+        <v>-0.1295</v>
       </c>
       <c r="J79" t="n">
-        <v>-3.576</v>
+        <v>-3.885</v>
       </c>
     </row>
     <row r="80">
@@ -4629,10 +4629,10 @@
         <v>0.89</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.153</v>
+        <v>-0.1643</v>
       </c>
       <c r="J80" t="n">
-        <v>-4.59</v>
+        <v>-4.929</v>
       </c>
     </row>
     <row r="81">
@@ -4669,10 +4669,10 @@
         <v>0.73</v>
       </c>
       <c r="I81" t="n">
-        <v>-0.3152</v>
+        <v>-0.3258</v>
       </c>
       <c r="J81" t="n">
-        <v>-9.456</v>
+        <v>-9.773999999999999</v>
       </c>
     </row>
     <row r="82">
@@ -4709,10 +4709,10 @@
         <v>1.61</v>
       </c>
       <c r="I82" t="n">
-        <v>1.2977</v>
+        <v>1.268</v>
       </c>
       <c r="J82" t="n">
-        <v>36.3356</v>
+        <v>35.504</v>
       </c>
     </row>
     <row r="83">
@@ -4749,10 +4749,10 @@
         <v>1.31</v>
       </c>
       <c r="I83" t="n">
-        <v>0.8343</v>
+        <v>0.7855</v>
       </c>
       <c r="J83" t="n">
-        <v>23.3604</v>
+        <v>21.994</v>
       </c>
     </row>
     <row r="84">
@@ -4789,10 +4789,10 @@
         <v>1.14</v>
       </c>
       <c r="I84" t="n">
-        <v>0.4216</v>
+        <v>0.4171</v>
       </c>
       <c r="J84" t="n">
-        <v>11.8048</v>
+        <v>11.6788</v>
       </c>
     </row>
     <row r="85">
@@ -4829,10 +4829,10 @@
         <v>0.86</v>
       </c>
       <c r="I85" t="n">
-        <v>-0.5017</v>
+        <v>-0.4727</v>
       </c>
       <c r="J85" t="n">
-        <v>-14.0476</v>
+        <v>-13.2356</v>
       </c>
     </row>
     <row r="86">
@@ -4869,10 +4869,10 @@
         <v>0.8</v>
       </c>
       <c r="I86" t="n">
-        <v>-0.6613</v>
+        <v>-0.6156</v>
       </c>
       <c r="J86" t="n">
-        <v>-18.5164</v>
+        <v>-17.2368</v>
       </c>
     </row>
     <row r="87">
@@ -4909,10 +4909,10 @@
         <v>1.23</v>
       </c>
       <c r="I87" t="n">
-        <v>0.5646</v>
+        <v>0.5367</v>
       </c>
       <c r="J87" t="n">
-        <v>15.8088</v>
+        <v>15.0276</v>
       </c>
     </row>
     <row r="88">
@@ -4949,10 +4949,10 @@
         <v>0.95</v>
       </c>
       <c r="I88" t="n">
-        <v>-0.0578</v>
+        <v>-0.0722</v>
       </c>
       <c r="J88" t="n">
-        <v>-1.6184</v>
+        <v>-2.0216</v>
       </c>
     </row>
     <row r="89">
@@ -4989,10 +4989,10 @@
         <v>0.92</v>
       </c>
       <c r="I89" t="n">
-        <v>-0.0948</v>
+        <v>-0.1107</v>
       </c>
       <c r="J89" t="n">
-        <v>-2.6544</v>
+        <v>-3.0996</v>
       </c>
     </row>
     <row r="90">
@@ -5029,10 +5029,10 @@
         <v>0.64</v>
       </c>
       <c r="I90" t="n">
-        <v>-0.3729</v>
+        <v>-0.3866</v>
       </c>
       <c r="J90" t="n">
-        <v>-10.4412</v>
+        <v>-10.8248</v>
       </c>
     </row>
     <row r="91">
@@ -5069,10 +5069,10 @@
         <v>0.46</v>
       </c>
       <c r="I91" t="n">
-        <v>-0.539</v>
+        <v>-0.5438</v>
       </c>
       <c r="J91" t="n">
-        <v>-15.092</v>
+        <v>-15.2264</v>
       </c>
     </row>
     <row r="92">
@@ -5109,10 +5109,10 @@
         <v>1.84</v>
       </c>
       <c r="I92" t="n">
-        <v>1.476</v>
+        <v>1.4732</v>
       </c>
       <c r="J92" t="n">
-        <v>26.568</v>
+        <v>26.5176</v>
       </c>
     </row>
     <row r="93">
@@ -5149,10 +5149,10 @@
         <v>1.63</v>
       </c>
       <c r="I93" t="n">
-        <v>1.2388</v>
+        <v>1.2206</v>
       </c>
       <c r="J93" t="n">
-        <v>22.2984</v>
+        <v>21.9708</v>
       </c>
     </row>
     <row r="94">
@@ -5189,10 +5189,10 @@
         <v>1.51</v>
       </c>
       <c r="I94" t="n">
-        <v>1.1024</v>
+        <v>1.0726</v>
       </c>
       <c r="J94" t="n">
-        <v>19.8432</v>
+        <v>19.3068</v>
       </c>
     </row>
     <row r="95">
@@ -5229,10 +5229,10 @@
         <v>1.45</v>
       </c>
       <c r="I95" t="n">
-        <v>1.0283</v>
+        <v>0.9868</v>
       </c>
       <c r="J95" t="n">
-        <v>18.5094</v>
+        <v>17.7624</v>
       </c>
     </row>
     <row r="96">
@@ -5269,10 +5269,10 @@
         <v>1.3</v>
       </c>
       <c r="I96" t="n">
-        <v>0.7271</v>
+        <v>0.7072000000000001</v>
       </c>
       <c r="J96" t="n">
-        <v>13.0878</v>
+        <v>12.7296</v>
       </c>
     </row>
     <row r="97">
@@ -5309,10 +5309,10 @@
         <v>0.73</v>
       </c>
       <c r="I97" t="n">
-        <v>-0.1817</v>
+        <v>-0.2212</v>
       </c>
       <c r="J97" t="n">
-        <v>-3.2706</v>
+        <v>-3.9816</v>
       </c>
     </row>
     <row r="98">
@@ -5349,10 +5349,10 @@
         <v>0.73</v>
       </c>
       <c r="I98" t="n">
-        <v>-0.1817</v>
+        <v>-0.2212</v>
       </c>
       <c r="J98" t="n">
-        <v>-3.2706</v>
+        <v>-3.9816</v>
       </c>
     </row>
     <row r="99">
@@ -5389,10 +5389,10 @@
         <v>0.45</v>
       </c>
       <c r="I99" t="n">
-        <v>-0.4821</v>
+        <v>-0.5007</v>
       </c>
       <c r="J99" t="n">
-        <v>-8.6778</v>
+        <v>-9.012600000000001</v>
       </c>
     </row>
     <row r="100">
@@ -5429,10 +5429,10 @@
         <v>0.23</v>
       </c>
       <c r="I100" t="n">
-        <v>-0.7010999999999999</v>
+        <v>-0.7003</v>
       </c>
       <c r="J100" t="n">
-        <v>-12.6198</v>
+        <v>-12.6054</v>
       </c>
     </row>
     <row r="101">
@@ -5469,10 +5469,10 @@
         <v>0.14</v>
       </c>
       <c r="I101" t="n">
-        <v>-0.7961</v>
+        <v>-0.7855</v>
       </c>
       <c r="J101" t="n">
-        <v>-14.3298</v>
+        <v>-14.139</v>
       </c>
     </row>
     <row r="102">
@@ -5509,10 +5509,10 @@
         <v>1.1</v>
       </c>
       <c r="I102" t="n">
-        <v>0.2719</v>
+        <v>0.2605</v>
       </c>
       <c r="J102" t="n">
-        <v>6.7975</v>
+        <v>6.5125</v>
       </c>
     </row>
     <row r="103">
@@ -5549,10 +5549,10 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="I103" t="n">
-        <v>-0.1984</v>
+        <v>-0.2189</v>
       </c>
       <c r="J103" t="n">
-        <v>-4.96</v>
+        <v>-5.4725</v>
       </c>
     </row>
     <row r="104">
@@ -5589,10 +5589,10 @@
         <v>0.72</v>
       </c>
       <c r="I104" t="n">
-        <v>-0.284</v>
+        <v>-0.3033</v>
       </c>
       <c r="J104" t="n">
-        <v>-7.1</v>
+        <v>-7.5825</v>
       </c>
     </row>
     <row r="105">
@@ -5629,10 +5629,10 @@
         <v>0.7</v>
       </c>
       <c r="I105" t="n">
-        <v>-0.3026</v>
+        <v>-0.3214</v>
       </c>
       <c r="J105" t="n">
-        <v>-7.565</v>
+        <v>-8.035</v>
       </c>
     </row>
     <row r="106">
@@ -5669,10 +5669,10 @@
         <v>0.39</v>
       </c>
       <c r="I106" t="n">
-        <v>-0.5913</v>
+        <v>-0.5943000000000001</v>
       </c>
       <c r="J106" t="n">
-        <v>-14.7825</v>
+        <v>-14.8575</v>
       </c>
     </row>
     <row r="107">
@@ -5709,10 +5709,10 @@
         <v>1.42</v>
       </c>
       <c r="I107" t="n">
-        <v>0.5387</v>
+        <v>0.545</v>
       </c>
       <c r="J107" t="n">
-        <v>13.4675</v>
+        <v>13.625</v>
       </c>
     </row>
     <row r="108">
@@ -5749,10 +5749,10 @@
         <v>1.3</v>
       </c>
       <c r="I108" t="n">
-        <v>0.4017</v>
+        <v>0.415</v>
       </c>
       <c r="J108" t="n">
-        <v>10.0425</v>
+        <v>10.375</v>
       </c>
     </row>
     <row r="109">
@@ -5789,10 +5789,10 @@
         <v>1.2</v>
       </c>
       <c r="I109" t="n">
-        <v>0.283</v>
+        <v>0.3</v>
       </c>
       <c r="J109" t="n">
-        <v>7.075</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="110">
@@ -5829,10 +5829,10 @@
         <v>1.04</v>
       </c>
       <c r="I110" t="n">
-        <v>0.0622</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="J110" t="n">
-        <v>1.555</v>
+        <v>1.9325</v>
       </c>
     </row>
     <row r="111">
@@ -5869,10 +5869,10 @@
         <v>0.95</v>
       </c>
       <c r="I111" t="n">
-        <v>-0.0946</v>
+        <v>-0.1006</v>
       </c>
       <c r="J111" t="n">
-        <v>-2.365</v>
+        <v>-2.515</v>
       </c>
     </row>
     <row r="112">
@@ -5909,10 +5909,10 @@
         <v>1.44</v>
       </c>
       <c r="I112" t="n">
-        <v>1.1253</v>
+        <v>1.0749</v>
       </c>
       <c r="J112" t="n">
-        <v>32.6337</v>
+        <v>31.1721</v>
       </c>
     </row>
     <row r="113">
@@ -5949,10 +5949,10 @@
         <v>0.99</v>
       </c>
       <c r="I113" t="n">
-        <v>-0.0527</v>
+        <v>-0.0582</v>
       </c>
       <c r="J113" t="n">
-        <v>-1.5283</v>
+        <v>-1.6878</v>
       </c>
     </row>
     <row r="114">
@@ -5989,10 +5989,10 @@
         <v>0.96</v>
       </c>
       <c r="I114" t="n">
-        <v>-0.1634</v>
+        <v>-0.1681</v>
       </c>
       <c r="J114" t="n">
-        <v>-4.7386</v>
+        <v>-4.8749</v>
       </c>
     </row>
     <row r="115">
@@ -6029,10 +6029,10 @@
         <v>0.86</v>
       </c>
       <c r="I115" t="n">
-        <v>-0.46</v>
+        <v>-0.4435</v>
       </c>
       <c r="J115" t="n">
-        <v>-13.34</v>
+        <v>-12.8615</v>
       </c>
     </row>
     <row r="116">
@@ -6069,10 +6069,10 @@
         <v>0.73</v>
       </c>
       <c r="I116" t="n">
-        <v>-0.7982</v>
+        <v>-0.7435</v>
       </c>
       <c r="J116" t="n">
-        <v>-23.1478</v>
+        <v>-21.5615</v>
       </c>
     </row>
     <row r="117">
@@ -6109,10 +6109,10 @@
         <v>1.18</v>
       </c>
       <c r="I117" t="n">
-        <v>0.4142</v>
+        <v>0.4084</v>
       </c>
       <c r="J117" t="n">
-        <v>12.0118</v>
+        <v>11.8436</v>
       </c>
     </row>
     <row r="118">
@@ -6149,10 +6149,10 @@
         <v>1.1</v>
       </c>
       <c r="I118" t="n">
-        <v>0.2567</v>
+        <v>0.26</v>
       </c>
       <c r="J118" t="n">
-        <v>7.4443</v>
+        <v>7.54</v>
       </c>
     </row>
     <row r="119">
@@ -6189,10 +6189,10 @@
         <v>1.01</v>
       </c>
       <c r="I119" t="n">
-        <v>0.0443</v>
+        <v>0.0481</v>
       </c>
       <c r="J119" t="n">
-        <v>1.2847</v>
+        <v>1.3949</v>
       </c>
     </row>
     <row r="120">
@@ -6229,10 +6229,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I120" t="n">
-        <v>-0.08450000000000001</v>
+        <v>-0.09619999999999999</v>
       </c>
       <c r="J120" t="n">
-        <v>-2.4505</v>
+        <v>-2.7898</v>
       </c>
     </row>
     <row r="121">
@@ -6269,10 +6269,10 @@
         <v>0.58</v>
       </c>
       <c r="I121" t="n">
-        <v>-0.4435</v>
+        <v>-0.4515</v>
       </c>
       <c r="J121" t="n">
-        <v>-12.8615</v>
+        <v>-13.0935</v>
       </c>
     </row>
     <row r="122">
@@ -6309,10 +6309,10 @@
         <v>1.21</v>
       </c>
       <c r="I122" t="n">
-        <v>0.4982</v>
+        <v>0.5479000000000001</v>
       </c>
       <c r="J122" t="n">
-        <v>13.4514</v>
+        <v>14.7933</v>
       </c>
     </row>
     <row r="123">
@@ -6349,10 +6349,10 @@
         <v>1.14</v>
       </c>
       <c r="I123" t="n">
-        <v>0.3923</v>
+        <v>0.4234</v>
       </c>
       <c r="J123" t="n">
-        <v>10.5921</v>
+        <v>11.4318</v>
       </c>
     </row>
     <row r="124">
@@ -6389,10 +6389,10 @@
         <v>1.13</v>
       </c>
       <c r="I124" t="n">
-        <v>0.3766</v>
+        <v>0.4003</v>
       </c>
       <c r="J124" t="n">
-        <v>10.1682</v>
+        <v>10.8081</v>
       </c>
     </row>
     <row r="125">
@@ -6429,10 +6429,10 @@
         <v>1.13</v>
       </c>
       <c r="I125" t="n">
-        <v>0.3766</v>
+        <v>0.4003</v>
       </c>
       <c r="J125" t="n">
-        <v>10.1682</v>
+        <v>10.8081</v>
       </c>
     </row>
     <row r="126">
@@ -6469,10 +6469,10 @@
         <v>0.82</v>
       </c>
       <c r="I126" t="n">
-        <v>-0.5936</v>
+        <v>-0.5583</v>
       </c>
       <c r="J126" t="n">
-        <v>-16.0272</v>
+        <v>-15.0741</v>
       </c>
     </row>
     <row r="127">
@@ -6509,10 +6509,10 @@
         <v>1.44</v>
       </c>
       <c r="I127" t="n">
-        <v>0.648</v>
+        <v>0.7207</v>
       </c>
       <c r="J127" t="n">
-        <v>17.496</v>
+        <v>19.4589</v>
       </c>
     </row>
     <row r="128">
@@ -6549,10 +6549,10 @@
         <v>1.16</v>
       </c>
       <c r="I128" t="n">
-        <v>0.3565</v>
+        <v>0.37</v>
       </c>
       <c r="J128" t="n">
-        <v>9.625500000000001</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="129">
@@ -6589,10 +6589,10 @@
         <v>1.06</v>
       </c>
       <c r="I129" t="n">
-        <v>0.1677</v>
+        <v>0.1744</v>
       </c>
       <c r="J129" t="n">
-        <v>4.5279</v>
+        <v>4.7088</v>
       </c>
     </row>
     <row r="130">
@@ -6629,10 +6629,10 @@
         <v>0.67</v>
       </c>
       <c r="I130" t="n">
-        <v>-0.3616</v>
+        <v>-0.3727</v>
       </c>
       <c r="J130" t="n">
-        <v>-9.763199999999999</v>
+        <v>-10.0629</v>
       </c>
     </row>
     <row r="131">
@@ -6669,10 +6669,10 @@
         <v>0.54</v>
       </c>
       <c r="I131" t="n">
-        <v>-0.481</v>
+        <v>-0.487</v>
       </c>
       <c r="J131" t="n">
-        <v>-12.987</v>
+        <v>-13.149</v>
       </c>
     </row>
     <row r="132">
@@ -6709,10 +6709,10 @@
         <v>1.44</v>
       </c>
       <c r="I132" t="n">
-        <v>0.7988</v>
+        <v>0.881</v>
       </c>
       <c r="J132" t="n">
-        <v>20.7688</v>
+        <v>22.906</v>
       </c>
     </row>
     <row r="133">
@@ -6749,10 +6749,10 @@
         <v>1.19</v>
       </c>
       <c r="I133" t="n">
-        <v>0.4565</v>
+        <v>0.5042</v>
       </c>
       <c r="J133" t="n">
-        <v>11.869</v>
+        <v>13.1092</v>
       </c>
     </row>
     <row r="134">
@@ -6789,10 +6789,10 @@
         <v>1.13</v>
       </c>
       <c r="I134" t="n">
-        <v>0.3684</v>
+        <v>0.391</v>
       </c>
       <c r="J134" t="n">
-        <v>9.5784</v>
+        <v>10.166</v>
       </c>
     </row>
     <row r="135">
@@ -6829,10 +6829,10 @@
         <v>1.12</v>
       </c>
       <c r="I135" t="n">
-        <v>0.3526</v>
+        <v>0.3666</v>
       </c>
       <c r="J135" t="n">
-        <v>9.1676</v>
+        <v>9.531599999999999</v>
       </c>
     </row>
     <row r="136">
@@ -6869,10 +6869,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I136" t="n">
-        <v>-0.2735</v>
+        <v>-0.2613</v>
       </c>
       <c r="J136" t="n">
-        <v>-7.111</v>
+        <v>-6.7938</v>
       </c>
     </row>
     <row r="137">
@@ -6909,10 +6909,10 @@
         <v>1.04</v>
       </c>
       <c r="I137" t="n">
-        <v>0.1696</v>
+        <v>0.1636</v>
       </c>
       <c r="J137" t="n">
-        <v>4.4096</v>
+        <v>4.2536</v>
       </c>
     </row>
     <row r="138">
@@ -6949,10 +6949,10 @@
         <v>0.89</v>
       </c>
       <c r="I138" t="n">
-        <v>-0.1269</v>
+        <v>-0.1442</v>
       </c>
       <c r="J138" t="n">
-        <v>-3.2994</v>
+        <v>-3.7492</v>
       </c>
     </row>
     <row r="139">
@@ -6989,10 +6989,10 @@
         <v>0.89</v>
       </c>
       <c r="I139" t="n">
-        <v>-0.1269</v>
+        <v>-0.1442</v>
       </c>
       <c r="J139" t="n">
-        <v>-3.2994</v>
+        <v>-3.7492</v>
       </c>
     </row>
     <row r="140">
@@ -7029,10 +7029,10 @@
         <v>0.75</v>
       </c>
       <c r="I140" t="n">
-        <v>-0.2663</v>
+        <v>-0.2838</v>
       </c>
       <c r="J140" t="n">
-        <v>-6.9238</v>
+        <v>-7.3788</v>
       </c>
     </row>
     <row r="141">
@@ -7069,10 +7069,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I141" t="n">
-        <v>-0.4455</v>
+        <v>-0.4561</v>
       </c>
       <c r="J141" t="n">
-        <v>-11.583</v>
+        <v>-11.8586</v>
       </c>
     </row>
     <row r="142">
@@ -7109,10 +7109,10 @@
         <v>1.66</v>
       </c>
       <c r="I142" t="n">
-        <v>1.0194</v>
+        <v>1.1276</v>
       </c>
       <c r="J142" t="n">
-        <v>18.3492</v>
+        <v>20.2968</v>
       </c>
     </row>
     <row r="143">
@@ -7149,10 +7149,10 @@
         <v>1.54</v>
       </c>
       <c r="I143" t="n">
-        <v>0.8768</v>
+        <v>0.9748</v>
       </c>
       <c r="J143" t="n">
-        <v>15.7824</v>
+        <v>17.5464</v>
       </c>
     </row>
     <row r="144">
@@ -7189,10 +7189,10 @@
         <v>1.42</v>
       </c>
       <c r="I144" t="n">
-        <v>0.7325</v>
+        <v>0.8178</v>
       </c>
       <c r="J144" t="n">
-        <v>13.185</v>
+        <v>14.7204</v>
       </c>
     </row>
     <row r="145">
@@ -7229,10 +7229,10 @@
         <v>1.31</v>
       </c>
       <c r="I145" t="n">
-        <v>0.5945</v>
+        <v>0.6656</v>
       </c>
       <c r="J145" t="n">
-        <v>10.701</v>
+        <v>11.9808</v>
       </c>
     </row>
     <row r="146">
@@ -7269,10 +7269,10 @@
         <v>1.13</v>
       </c>
       <c r="I146" t="n">
-        <v>0.333</v>
+        <v>0.3526</v>
       </c>
       <c r="J146" t="n">
-        <v>5.994</v>
+        <v>6.3468</v>
       </c>
     </row>
     <row r="147">
@@ -7309,10 +7309,10 @@
         <v>0.87</v>
       </c>
       <c r="I147" t="n">
-        <v>-0.0732</v>
+        <v>-0.107</v>
       </c>
       <c r="J147" t="n">
-        <v>-1.3176</v>
+        <v>-1.926</v>
       </c>
     </row>
     <row r="148">
@@ -7349,10 +7349,10 @@
         <v>0.7</v>
       </c>
       <c r="I148" t="n">
-        <v>-0.2685</v>
+        <v>-0.2951</v>
       </c>
       <c r="J148" t="n">
-        <v>-4.833</v>
+        <v>-5.3118</v>
       </c>
     </row>
     <row r="149">
@@ -7389,10 +7389,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I149" t="n">
-        <v>-0.4038</v>
+        <v>-0.4236</v>
       </c>
       <c r="J149" t="n">
-        <v>-7.2684</v>
+        <v>-7.6248</v>
       </c>
     </row>
     <row r="150">
@@ -7429,10 +7429,10 @@
         <v>0.35</v>
       </c>
       <c r="I150" t="n">
-        <v>-0.6019</v>
+        <v>-0.6077</v>
       </c>
       <c r="J150" t="n">
-        <v>-10.8342</v>
+        <v>-10.9386</v>
       </c>
     </row>
     <row r="151">
@@ -7469,10 +7469,10 @@
         <v>0.35</v>
       </c>
       <c r="I151" t="n">
-        <v>-0.6019</v>
+        <v>-0.6077</v>
       </c>
       <c r="J151" t="n">
-        <v>-10.8342</v>
+        <v>-10.9386</v>
       </c>
     </row>
     <row r="152">
@@ -7509,10 +7509,10 @@
         <v>1.29</v>
       </c>
       <c r="I152" t="n">
-        <v>0.5905</v>
+        <v>0.6555</v>
       </c>
       <c r="J152" t="n">
-        <v>12.991</v>
+        <v>14.421</v>
       </c>
     </row>
     <row r="153">
@@ -7549,10 +7549,10 @@
         <v>1.29</v>
       </c>
       <c r="I153" t="n">
-        <v>0.5905</v>
+        <v>0.6555</v>
       </c>
       <c r="J153" t="n">
-        <v>12.991</v>
+        <v>14.421</v>
       </c>
     </row>
     <row r="154">
@@ -7589,10 +7589,10 @@
         <v>1.18</v>
       </c>
       <c r="I154" t="n">
-        <v>0.4387</v>
+        <v>0.4851</v>
       </c>
       <c r="J154" t="n">
-        <v>9.651400000000001</v>
+        <v>10.6722</v>
       </c>
     </row>
     <row r="155">
@@ -7629,10 +7629,10 @@
         <v>1.17</v>
       </c>
       <c r="I155" t="n">
-        <v>0.4242</v>
+        <v>0.4684</v>
       </c>
       <c r="J155" t="n">
-        <v>9.3324</v>
+        <v>10.3048</v>
       </c>
     </row>
     <row r="156">
@@ -7669,10 +7669,10 @@
         <v>1.09</v>
       </c>
       <c r="I156" t="n">
-        <v>0.273</v>
+        <v>0.2832</v>
       </c>
       <c r="J156" t="n">
-        <v>6.006</v>
+        <v>6.2304</v>
       </c>
     </row>
     <row r="157">
@@ -7709,10 +7709,10 @@
         <v>0.82</v>
       </c>
       <c r="I157" t="n">
-        <v>-0.1812</v>
+        <v>-0.2033</v>
       </c>
       <c r="J157" t="n">
-        <v>-3.9864</v>
+        <v>-4.4726</v>
       </c>
     </row>
     <row r="158">
@@ -7749,10 +7749,10 @@
         <v>0.8</v>
       </c>
       <c r="I158" t="n">
-        <v>-0.2022</v>
+        <v>-0.2241</v>
       </c>
       <c r="J158" t="n">
-        <v>-4.4484</v>
+        <v>-4.9302</v>
       </c>
     </row>
     <row r="159">
@@ -7789,10 +7789,10 @@
         <v>0.75</v>
       </c>
       <c r="I159" t="n">
-        <v>-0.2525</v>
+        <v>-0.2733</v>
       </c>
       <c r="J159" t="n">
-        <v>-5.555</v>
+        <v>-6.0126</v>
       </c>
     </row>
     <row r="160">
@@ -7829,10 +7829,10 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="I160" t="n">
-        <v>-0.3073</v>
+        <v>-0.327</v>
       </c>
       <c r="J160" t="n">
-        <v>-6.7606</v>
+        <v>-7.194</v>
       </c>
     </row>
     <row r="161">
@@ -7869,10 +7869,10 @@
         <v>0.49</v>
       </c>
       <c r="I161" t="n">
-        <v>-0.4937</v>
+        <v>-0.504</v>
       </c>
       <c r="J161" t="n">
-        <v>-10.8614</v>
+        <v>-11.088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>